<commit_message>
Update translation report with 2026-03-13 data
</commit_message>
<xml_diff>
--- a/reports/translation_jobs_all_days.xlsx
+++ b/reports/translation_jobs_all_days.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Translation Jobs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors by Date" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RMTranslationRequest" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Translation Jobs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Errors by Date" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="RMTranslationRequest" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Translation Jobs'!$A$1:$AD$244</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Translation Jobs'!$A$1:$AD$250</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD244"/>
+  <dimension ref="A1:AD250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30602,8 +30602,764 @@
       <c r="AC244" s="2" t="inlineStr"/>
       <c r="AD244" s="2" t="inlineStr"/>
     </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B245" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="C245" s="2" t="inlineStr">
+        <is>
+          <t>translationjob42</t>
+        </is>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>Ana Ai Translation Project</t>
+        </is>
+      </c>
+      <c r="E245" s="2" t="inlineStr">
+        <is>
+          <t>DE-DE</t>
+        </is>
+      </c>
+      <c r="F245" s="2" t="inlineStr">
+        <is>
+          <t>es_es</t>
+        </is>
+      </c>
+      <c r="G245" s="2" t="inlineStr">
+        <is>
+          <t>rmcf-ai-translatorion-connector</t>
+        </is>
+      </c>
+      <c r="H245" s="2" t="inlineStr">
+        <is>
+          <t>MACHINE_TRANSLATION</t>
+        </is>
+      </c>
+      <c r="I245" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J245" s="2" t="inlineStr">
+        <is>
+          <t>18:28:16.617</t>
+        </is>
+      </c>
+      <c r="K245" s="2" t="inlineStr">
+        <is>
+          <t>18:28:16.637</t>
+        </is>
+      </c>
+      <c r="L245" s="2" t="inlineStr">
+        <is>
+          <t>18:28:17.068</t>
+        </is>
+      </c>
+      <c r="M245" s="2" t="inlineStr">
+        <is>
+          <t>18:28:22.260</t>
+        </is>
+      </c>
+      <c r="N245" s="2" t="inlineStr">
+        <is>
+          <t>18:28:22.338</t>
+        </is>
+      </c>
+      <c r="O245" s="2" t="inlineStr">
+        <is>
+          <t>18:28:22.414</t>
+        </is>
+      </c>
+      <c r="P245" s="2" t="n">
+        <v>431</v>
+      </c>
+      <c r="Q245" s="2" t="inlineStr">
+        <is>
+          <t>0.4s</t>
+        </is>
+      </c>
+      <c r="R245" s="2" t="n">
+        <v>5643</v>
+      </c>
+      <c r="S245" s="2" t="inlineStr">
+        <is>
+          <t>5.6s</t>
+        </is>
+      </c>
+      <c r="T245" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="U245" s="2" t="inlineStr">
+        <is>
+          <t>0.1s</t>
+        </is>
+      </c>
+      <c r="V245" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="W245" s="2" t="inlineStr">
+        <is>
+          <t>0.1s</t>
+        </is>
+      </c>
+      <c r="X245" s="2" t="n">
+        <v>5797</v>
+      </c>
+      <c r="Y245" s="2" t="inlineStr">
+        <is>
+          <t>5.8s</t>
+        </is>
+      </c>
+      <c r="Z245" s="2" t="inlineStr">
+        <is>
+          <t>page:0, asset:0, contentFragment:1, i18nComponentStringDict:0, assetMetaData:0, tagMetadata:0, tag:0</t>
+        </is>
+      </c>
+      <c r="AA245" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB245" s="2" t="inlineStr"/>
+      <c r="AC245" s="2" t="inlineStr"/>
+      <c r="AD245" s="2" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="C246" s="2" t="inlineStr">
+        <is>
+          <t>translationjob43</t>
+        </is>
+      </c>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>Ana Ai Translation Project</t>
+        </is>
+      </c>
+      <c r="E246" s="2" t="inlineStr">
+        <is>
+          <t>PT-PT</t>
+        </is>
+      </c>
+      <c r="F246" s="2" t="inlineStr">
+        <is>
+          <t>es_es</t>
+        </is>
+      </c>
+      <c r="G246" s="2" t="inlineStr">
+        <is>
+          <t>rmcf-ai-translatorion-connector</t>
+        </is>
+      </c>
+      <c r="H246" s="2" t="inlineStr">
+        <is>
+          <t>MACHINE_TRANSLATION</t>
+        </is>
+      </c>
+      <c r="I246" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J246" s="2" t="inlineStr">
+        <is>
+          <t>18:28:22.589</t>
+        </is>
+      </c>
+      <c r="K246" s="2" t="inlineStr">
+        <is>
+          <t>18:28:22.609</t>
+        </is>
+      </c>
+      <c r="L246" s="2" t="inlineStr">
+        <is>
+          <t>18:28:22.940</t>
+        </is>
+      </c>
+      <c r="M246" s="2" t="inlineStr">
+        <is>
+          <t>18:28:26.629</t>
+        </is>
+      </c>
+      <c r="N246" s="2" t="inlineStr">
+        <is>
+          <t>18:28:26.688</t>
+        </is>
+      </c>
+      <c r="O246" s="2" t="inlineStr">
+        <is>
+          <t>18:28:26.753</t>
+        </is>
+      </c>
+      <c r="P246" s="2" t="n">
+        <v>331</v>
+      </c>
+      <c r="Q246" s="2" t="inlineStr">
+        <is>
+          <t>0.3s</t>
+        </is>
+      </c>
+      <c r="R246" s="2" t="n">
+        <v>4040</v>
+      </c>
+      <c r="S246" s="2" t="inlineStr">
+        <is>
+          <t>4.0s</t>
+        </is>
+      </c>
+      <c r="T246" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="U246" s="2" t="inlineStr">
+        <is>
+          <t>0.1s</t>
+        </is>
+      </c>
+      <c r="V246" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="W246" s="2" t="inlineStr">
+        <is>
+          <t>0.1s</t>
+        </is>
+      </c>
+      <c r="X246" s="2" t="n">
+        <v>4164</v>
+      </c>
+      <c r="Y246" s="2" t="inlineStr">
+        <is>
+          <t>4.2s</t>
+        </is>
+      </c>
+      <c r="Z246" s="2" t="inlineStr">
+        <is>
+          <t>page:0, asset:0, contentFragment:1, i18nComponentStringDict:0, assetMetaData:0, tagMetadata:0, tag:0</t>
+        </is>
+      </c>
+      <c r="AA246" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB246" s="2" t="inlineStr"/>
+      <c r="AC246" s="2" t="inlineStr"/>
+      <c r="AD246" s="2" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B247" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="C247" s="2" t="inlineStr">
+        <is>
+          <t>translationjob44</t>
+        </is>
+      </c>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>Ana Ai Translation Project</t>
+        </is>
+      </c>
+      <c r="E247" s="2" t="inlineStr">
+        <is>
+          <t>EN-US</t>
+        </is>
+      </c>
+      <c r="F247" s="2" t="inlineStr">
+        <is>
+          <t>es_es</t>
+        </is>
+      </c>
+      <c r="G247" s="2" t="inlineStr">
+        <is>
+          <t>rmcf-ai-translatorion-connector</t>
+        </is>
+      </c>
+      <c r="H247" s="2" t="inlineStr">
+        <is>
+          <t>MACHINE_TRANSLATION</t>
+        </is>
+      </c>
+      <c r="I247" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J247" s="2" t="inlineStr">
+        <is>
+          <t>18:28:26.915</t>
+        </is>
+      </c>
+      <c r="K247" s="2" t="inlineStr">
+        <is>
+          <t>18:28:26.932</t>
+        </is>
+      </c>
+      <c r="L247" s="2" t="inlineStr">
+        <is>
+          <t>18:28:27.228</t>
+        </is>
+      </c>
+      <c r="M247" s="2" t="inlineStr">
+        <is>
+          <t>18:28:32.377</t>
+        </is>
+      </c>
+      <c r="N247" s="2" t="inlineStr">
+        <is>
+          <t>18:28:32.443</t>
+        </is>
+      </c>
+      <c r="O247" s="2" t="inlineStr">
+        <is>
+          <t>18:28:32.506</t>
+        </is>
+      </c>
+      <c r="P247" s="2" t="n">
+        <v>296</v>
+      </c>
+      <c r="Q247" s="2" t="inlineStr">
+        <is>
+          <t>0.3s</t>
+        </is>
+      </c>
+      <c r="R247" s="2" t="n">
+        <v>5462</v>
+      </c>
+      <c r="S247" s="2" t="inlineStr">
+        <is>
+          <t>5.5s</t>
+        </is>
+      </c>
+      <c r="T247" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="U247" s="2" t="inlineStr">
+        <is>
+          <t>0.1s</t>
+        </is>
+      </c>
+      <c r="V247" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="W247" s="2" t="inlineStr">
+        <is>
+          <t>0.1s</t>
+        </is>
+      </c>
+      <c r="X247" s="2" t="n">
+        <v>5591</v>
+      </c>
+      <c r="Y247" s="2" t="inlineStr">
+        <is>
+          <t>5.6s</t>
+        </is>
+      </c>
+      <c r="Z247" s="2" t="inlineStr">
+        <is>
+          <t>page:0, asset:0, contentFragment:1, i18nComponentStringDict:0, assetMetaData:0, tagMetadata:0, tag:0</t>
+        </is>
+      </c>
+      <c r="AA247" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB247" s="2" t="inlineStr"/>
+      <c r="AC247" s="2" t="inlineStr"/>
+      <c r="AD247" s="2" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="C248" s="2" t="inlineStr">
+        <is>
+          <t>translationjob45</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>Ana Ai Translation Project</t>
+        </is>
+      </c>
+      <c r="E248" s="2" t="inlineStr">
+        <is>
+          <t>AR-AE</t>
+        </is>
+      </c>
+      <c r="F248" s="2" t="inlineStr">
+        <is>
+          <t>es_es</t>
+        </is>
+      </c>
+      <c r="G248" s="2" t="inlineStr">
+        <is>
+          <t>rmcf-ai-translatorion-connector</t>
+        </is>
+      </c>
+      <c r="H248" s="2" t="inlineStr">
+        <is>
+          <t>MACHINE_TRANSLATION</t>
+        </is>
+      </c>
+      <c r="I248" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J248" s="2" t="inlineStr">
+        <is>
+          <t>18:28:32.712</t>
+        </is>
+      </c>
+      <c r="K248" s="2" t="inlineStr">
+        <is>
+          <t>18:28:32.782</t>
+        </is>
+      </c>
+      <c r="L248" s="2" t="inlineStr">
+        <is>
+          <t>18:28:33.018</t>
+        </is>
+      </c>
+      <c r="M248" s="2" t="inlineStr">
+        <is>
+          <t>18:28:36.608</t>
+        </is>
+      </c>
+      <c r="N248" s="2" t="inlineStr">
+        <is>
+          <t>18:28:36.654</t>
+        </is>
+      </c>
+      <c r="O248" s="2" t="inlineStr">
+        <is>
+          <t>18:28:36.717</t>
+        </is>
+      </c>
+      <c r="P248" s="2" t="n">
+        <v>236</v>
+      </c>
+      <c r="Q248" s="2" t="inlineStr">
+        <is>
+          <t>0.2s</t>
+        </is>
+      </c>
+      <c r="R248" s="2" t="n">
+        <v>3896</v>
+      </c>
+      <c r="S248" s="2" t="inlineStr">
+        <is>
+          <t>3.9s</t>
+        </is>
+      </c>
+      <c r="T248" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="U248" s="2" t="inlineStr">
+        <is>
+          <t>0.0s</t>
+        </is>
+      </c>
+      <c r="V248" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="W248" s="2" t="inlineStr">
+        <is>
+          <t>0.1s</t>
+        </is>
+      </c>
+      <c r="X248" s="2" t="n">
+        <v>4005</v>
+      </c>
+      <c r="Y248" s="2" t="inlineStr">
+        <is>
+          <t>4.0s</t>
+        </is>
+      </c>
+      <c r="Z248" s="2" t="inlineStr">
+        <is>
+          <t>page:0, asset:0, contentFragment:1, i18nComponentStringDict:0, assetMetaData:0, tagMetadata:0, tag:0</t>
+        </is>
+      </c>
+      <c r="AA248" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB248" s="2" t="inlineStr"/>
+      <c r="AC248" s="2" t="inlineStr"/>
+      <c r="AD248" s="2" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="C249" s="2" t="inlineStr">
+        <is>
+          <t>translationjob46</t>
+        </is>
+      </c>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>Ana Ai Translation Project</t>
+        </is>
+      </c>
+      <c r="E249" s="2" t="inlineStr">
+        <is>
+          <t>FR-FR</t>
+        </is>
+      </c>
+      <c r="F249" s="2" t="inlineStr">
+        <is>
+          <t>es_es</t>
+        </is>
+      </c>
+      <c r="G249" s="2" t="inlineStr">
+        <is>
+          <t>rmcf-ai-translatorion-connector</t>
+        </is>
+      </c>
+      <c r="H249" s="2" t="inlineStr">
+        <is>
+          <t>MACHINE_TRANSLATION</t>
+        </is>
+      </c>
+      <c r="I249" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J249" s="2" t="inlineStr">
+        <is>
+          <t>18:28:36.935</t>
+        </is>
+      </c>
+      <c r="K249" s="2" t="inlineStr">
+        <is>
+          <t>18:28:36.953</t>
+        </is>
+      </c>
+      <c r="L249" s="2" t="inlineStr">
+        <is>
+          <t>18:28:37.273</t>
+        </is>
+      </c>
+      <c r="M249" s="2" t="inlineStr">
+        <is>
+          <t>18:28:40.188</t>
+        </is>
+      </c>
+      <c r="N249" s="2" t="inlineStr">
+        <is>
+          <t>18:28:40.258</t>
+        </is>
+      </c>
+      <c r="O249" s="2" t="inlineStr">
+        <is>
+          <t>18:28:40.313</t>
+        </is>
+      </c>
+      <c r="P249" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="Q249" s="2" t="inlineStr">
+        <is>
+          <t>0.3s</t>
+        </is>
+      </c>
+      <c r="R249" s="2" t="n">
+        <v>3253</v>
+      </c>
+      <c r="S249" s="2" t="inlineStr">
+        <is>
+          <t>3.3s</t>
+        </is>
+      </c>
+      <c r="T249" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="U249" s="2" t="inlineStr">
+        <is>
+          <t>0.1s</t>
+        </is>
+      </c>
+      <c r="V249" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="W249" s="2" t="inlineStr">
+        <is>
+          <t>0.1s</t>
+        </is>
+      </c>
+      <c r="X249" s="2" t="n">
+        <v>3378</v>
+      </c>
+      <c r="Y249" s="2" t="inlineStr">
+        <is>
+          <t>3.4s</t>
+        </is>
+      </c>
+      <c r="Z249" s="2" t="inlineStr">
+        <is>
+          <t>page:0, asset:0, contentFragment:1, i18nComponentStringDict:0, assetMetaData:0, tagMetadata:0, tag:0</t>
+        </is>
+      </c>
+      <c r="AA249" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB249" s="2" t="inlineStr"/>
+      <c r="AC249" s="2" t="inlineStr"/>
+      <c r="AD249" s="2" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="C250" s="2" t="inlineStr">
+        <is>
+          <t>translationjob47</t>
+        </is>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>Ana Ai Translation Project</t>
+        </is>
+      </c>
+      <c r="E250" s="2" t="inlineStr">
+        <is>
+          <t>JA-JP</t>
+        </is>
+      </c>
+      <c r="F250" s="2" t="inlineStr">
+        <is>
+          <t>es_es</t>
+        </is>
+      </c>
+      <c r="G250" s="2" t="inlineStr">
+        <is>
+          <t>rmcf-ai-translatorion-connector</t>
+        </is>
+      </c>
+      <c r="H250" s="2" t="inlineStr">
+        <is>
+          <t>MACHINE_TRANSLATION</t>
+        </is>
+      </c>
+      <c r="I250" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J250" s="2" t="inlineStr">
+        <is>
+          <t>18:28:40.493</t>
+        </is>
+      </c>
+      <c r="K250" s="2" t="inlineStr">
+        <is>
+          <t>18:28:40.512</t>
+        </is>
+      </c>
+      <c r="L250" s="2" t="inlineStr">
+        <is>
+          <t>18:28:40.704</t>
+        </is>
+      </c>
+      <c r="M250" s="2" t="inlineStr">
+        <is>
+          <t>18:28:45.261</t>
+        </is>
+      </c>
+      <c r="N250" s="2" t="inlineStr">
+        <is>
+          <t>18:28:45.314</t>
+        </is>
+      </c>
+      <c r="O250" s="2" t="inlineStr">
+        <is>
+          <t>18:28:45.398</t>
+        </is>
+      </c>
+      <c r="P250" s="2" t="n">
+        <v>192</v>
+      </c>
+      <c r="Q250" s="2" t="inlineStr">
+        <is>
+          <t>0.2s</t>
+        </is>
+      </c>
+      <c r="R250" s="2" t="n">
+        <v>4768</v>
+      </c>
+      <c r="S250" s="2" t="inlineStr">
+        <is>
+          <t>4.8s</t>
+        </is>
+      </c>
+      <c r="T250" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="U250" s="2" t="inlineStr">
+        <is>
+          <t>0.1s</t>
+        </is>
+      </c>
+      <c r="V250" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="W250" s="2" t="inlineStr">
+        <is>
+          <t>0.1s</t>
+        </is>
+      </c>
+      <c r="X250" s="2" t="n">
+        <v>4905</v>
+      </c>
+      <c r="Y250" s="2" t="inlineStr">
+        <is>
+          <t>4.9s</t>
+        </is>
+      </c>
+      <c r="Z250" s="2" t="inlineStr">
+        <is>
+          <t>page:0, asset:0, contentFragment:1, i18nComponentStringDict:0, assetMetaData:0, tagMetadata:0, tag:0</t>
+        </is>
+      </c>
+      <c r="AA250" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB250" s="2" t="inlineStr"/>
+      <c r="AC250" s="2" t="inlineStr"/>
+      <c r="AD250" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AD244"/>
+  <autoFilter ref="A1:AD250"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -30768,10 +31524,10 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>0</v>
@@ -30854,7 +31610,7 @@
         <v>662</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3">
@@ -30950,7 +31706,7 @@
         <v>45485</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>44689</v>
+        <v>44773</v>
       </c>
     </row>
     <row r="10">
@@ -30964,7 +31720,7 @@
         <v>227</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>22332</v>
+        <v>22408</v>
       </c>
     </row>
     <row r="11">
@@ -30992,7 +31748,7 @@
         <v>808</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>308</v>
+        <v>350</v>
       </c>
     </row>
     <row r="13">
@@ -31006,7 +31762,7 @@
         <v>578</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>176</v>
+        <v>188</v>
       </c>
     </row>
     <row r="14">
@@ -31140,16 +31896,16 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>126</v>
+        <v>144</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="F4" s="6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Update translation report with 2026-03-17 data
</commit_message>
<xml_diff>
--- a/reports/translation_jobs_all_days.xlsx
+++ b/reports/translation_jobs_all_days.xlsx
@@ -13,7 +13,7 @@
     <sheet name="RMTranslationRequest" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Translation Jobs'!$A$1:$AD$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Translation Jobs'!$A$1:$AD$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,8 +36,12 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Consolas"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -50,8 +54,20 @@
         <bgColor rgb="002E3345"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+        <bgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+        <bgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -59,16 +75,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD1"/>
+  <dimension ref="A1:AD7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -621,8 +654,764 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>translationjob142</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Ignacio Ai Translation Project</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>DE-DE</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>es_es</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>rmcf-ai-translatorion-connector</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>MACHINE_TRANSLATION</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>01:35:07.803</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>01:35:07.818</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>01:35:24.456</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>01:35:45.003</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>01:35:45.041</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>01:35:45.219</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>16638</v>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>16.6s</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="n">
+        <v>37200</v>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>37.2s</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>0.0s</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="n">
+        <v>178</v>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>0.2s</t>
+        </is>
+      </c>
+      <c r="X2" s="2" t="n">
+        <v>37416</v>
+      </c>
+      <c r="Y2" s="2" t="inlineStr">
+        <is>
+          <t>37.4s</t>
+        </is>
+      </c>
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t>page:0, asset:0, contentFragment:4, i18nComponentStringDict:0, assetMetaData:0, tagMetadata:0, tag:0</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AC2" s="2" t="inlineStr"/>
+      <c r="AD2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>translationjob143</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Ignacio Ai Translation Project</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>PT-PT</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>es_es</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>rmcf-ai-translatorion-connector</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>MACHINE_TRANSLATION</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>01:35:55.782</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>01:35:55.793</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>01:36:12.977</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>01:36:34.213</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>01:36:34.251</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>01:36:34.424</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>17184</v>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>17.2s</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>38431</v>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>38.4s</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>0.0s</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="n">
+        <v>173</v>
+      </c>
+      <c r="W3" s="2" t="inlineStr">
+        <is>
+          <t>0.2s</t>
+        </is>
+      </c>
+      <c r="X3" s="2" t="n">
+        <v>38642</v>
+      </c>
+      <c r="Y3" s="2" t="inlineStr">
+        <is>
+          <t>38.6s</t>
+        </is>
+      </c>
+      <c r="Z3" s="2" t="inlineStr">
+        <is>
+          <t>page:0, asset:0, contentFragment:4, i18nComponentStringDict:0, assetMetaData:0, tagMetadata:0, tag:0</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>translationjob144</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Ignacio Ai Translation Project</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>EN-US</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>es_es</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>rmcf-ai-translatorion-connector</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>MACHINE_TRANSLATION</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>01:36:47.251</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>01:36:47.264</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>01:37:44.967</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>01:38:06.891</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>01:38:06.950</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>01:38:07.195</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>57703</v>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>57.7s</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>79640</v>
+      </c>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>1m 19.6s</t>
+        </is>
+      </c>
+      <c r="T4" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>0.1s</t>
+        </is>
+      </c>
+      <c r="V4" s="2" t="n">
+        <v>245</v>
+      </c>
+      <c r="W4" s="2" t="inlineStr">
+        <is>
+          <t>0.2s</t>
+        </is>
+      </c>
+      <c r="X4" s="2" t="n">
+        <v>79944</v>
+      </c>
+      <c r="Y4" s="2" t="inlineStr">
+        <is>
+          <t>1m 19.9s</t>
+        </is>
+      </c>
+      <c r="Z4" s="2" t="inlineStr">
+        <is>
+          <t>page:0, asset:0, contentFragment:5, i18nComponentStringDict:0, assetMetaData:0, tagMetadata:0, tag:0</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>translationjob145</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Ignacio Ai Translation Project</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>AR-AE</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>es_es</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>rmcf-ai-translatorion-connector</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>MACHINE_TRANSLATION</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>01:38:24.864</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>01:38:24.877</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>01:38:40.797</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>01:38:59.982</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>01:39:00.021</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>01:39:00.187</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>15920</v>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>15.9s</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>35118</v>
+      </c>
+      <c r="S5" s="2" t="inlineStr">
+        <is>
+          <t>35.1s</t>
+        </is>
+      </c>
+      <c r="T5" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="U5" s="2" t="inlineStr">
+        <is>
+          <t>0.0s</t>
+        </is>
+      </c>
+      <c r="V5" s="2" t="n">
+        <v>166</v>
+      </c>
+      <c r="W5" s="2" t="inlineStr">
+        <is>
+          <t>0.2s</t>
+        </is>
+      </c>
+      <c r="X5" s="2" t="n">
+        <v>35323</v>
+      </c>
+      <c r="Y5" s="2" t="inlineStr">
+        <is>
+          <t>35.3s</t>
+        </is>
+      </c>
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>page:0, asset:0, contentFragment:4, i18nComponentStringDict:0, assetMetaData:0, tagMetadata:0, tag:0</t>
+        </is>
+      </c>
+      <c r="AA5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>translationjob146</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Ignacio Ai Translation Project</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>FR-FR</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>es_es</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>rmcf-ai-translatorion-connector</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>MACHINE_TRANSLATION</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>01:39:11.457</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>01:39:11.470</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>01:39:27.446</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>01:39:53.430</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>01:39:53.473</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>01:39:53.632</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>15976</v>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>16.0s</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>41973</v>
+      </c>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>42.0s</t>
+        </is>
+      </c>
+      <c r="T6" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>0.0s</t>
+        </is>
+      </c>
+      <c r="V6" s="2" t="n">
+        <v>159</v>
+      </c>
+      <c r="W6" s="2" t="inlineStr">
+        <is>
+          <t>0.2s</t>
+        </is>
+      </c>
+      <c r="X6" s="2" t="n">
+        <v>42175</v>
+      </c>
+      <c r="Y6" s="2" t="inlineStr">
+        <is>
+          <t>42.2s</t>
+        </is>
+      </c>
+      <c r="Z6" s="2" t="inlineStr">
+        <is>
+          <t>page:0, asset:0, contentFragment:4, i18nComponentStringDict:0, assetMetaData:0, tagMetadata:0, tag:0</t>
+        </is>
+      </c>
+      <c r="AA6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>translationjob147</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Ignacio Ai Translation Project</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>JA-JP</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>es_es</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>rmcf-ai-translatorion-connector</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>MACHINE_TRANSLATION</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>01:40:04.332</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>01:40:04.345</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>01:40:22.123</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>01:40:46.786</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>01:40:46.820</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>01:40:46.991</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>17778</v>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>17.8s</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="n">
+        <v>42454</v>
+      </c>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>42.5s</t>
+        </is>
+      </c>
+      <c r="T7" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>0.0s</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="n">
+        <v>171</v>
+      </c>
+      <c r="W7" s="2" t="inlineStr">
+        <is>
+          <t>0.2s</t>
+        </is>
+      </c>
+      <c r="X7" s="2" t="n">
+        <v>42659</v>
+      </c>
+      <c r="Y7" s="2" t="inlineStr">
+        <is>
+          <t>42.7s</t>
+        </is>
+      </c>
+      <c r="Z7" s="2" t="inlineStr">
+        <is>
+          <t>page:0, asset:0, contentFragment:4, i18nComponentStringDict:0, assetMetaData:0, tagMetadata:0, tag:0</t>
+        </is>
+      </c>
+      <c r="AA7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AD1"/>
+  <autoFilter ref="A1:AD7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -633,7 +1422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -649,54 +1438,94 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Total Jobs</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Errors</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Stuck</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Retried</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Avg Duration</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Min Duration</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Max Duration</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>46.0s</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>35.3s</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>1m 19.9s</t>
         </is>
       </c>
     </row>
@@ -711,17 +1540,93 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Error Category</t>
         </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Language copy not found</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>95728</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>TicketAssemblyTranslationServiceImpl</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>ReplicationSquadListener</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>30119</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>ResourceUtils commit</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>1360</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>LockUtil contention</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>TranslateHrefAttributes</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Error executing workflow</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -735,7 +1640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -748,40 +1653,65 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Total Entries</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Init</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Obtained</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Expires</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Errors</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Token Size Entries</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update translation report with 2026-04-14 data
</commit_message>
<xml_diff>
--- a/reports/translation_jobs_all_days.xlsx
+++ b/reports/translation_jobs_all_days.xlsx
@@ -13,7 +13,7 @@
     <sheet name="RMTranslationRequest" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Translation Jobs'!$A$1:$AD$245</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Translation Jobs'!$A$1:$AI$245</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD245"/>
+  <dimension ref="A1:AI245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -514,6 +514,11 @@
     <col width="12" customWidth="1" min="28" max="28"/>
     <col width="12" customWidth="1" min="29" max="29"/>
     <col width="16" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="17" customWidth="1" min="32" max="32"/>
+    <col width="21" customWidth="1" min="33" max="33"/>
+    <col width="16" customWidth="1" min="34" max="34"/>
+    <col width="20" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -667,6 +672,31 @@
           <t>Retry Detail</t>
         </is>
       </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>API Requests</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Prompt Tokens</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Completion Tokens</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Total Tokens</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Avg Latency (ms)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -793,6 +823,11 @@
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="inlineStr"/>
       <c r="AD2" s="2" t="inlineStr"/>
+      <c r="AE2" s="2" t="inlineStr"/>
+      <c r="AF2" s="2" t="inlineStr"/>
+      <c r="AG2" s="2" t="inlineStr"/>
+      <c r="AH2" s="2" t="inlineStr"/>
+      <c r="AI2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -919,6 +954,11 @@
       <c r="AB3" s="2" t="inlineStr"/>
       <c r="AC3" s="2" t="inlineStr"/>
       <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr"/>
+      <c r="AG3" s="2" t="inlineStr"/>
+      <c r="AH3" s="2" t="inlineStr"/>
+      <c r="AI3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1045,6 +1085,11 @@
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr"/>
       <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr"/>
+      <c r="AG4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AI4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1171,6 +1216,11 @@
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr"/>
       <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr"/>
+      <c r="AG5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AI5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1297,6 +1347,11 @@
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr"/>
       <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="AF6" s="2" t="inlineStr"/>
+      <c r="AG6" s="2" t="inlineStr"/>
+      <c r="AH6" s="2" t="inlineStr"/>
+      <c r="AI6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1423,6 +1478,11 @@
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr"/>
       <c r="AD7" s="2" t="inlineStr"/>
+      <c r="AE7" s="2" t="inlineStr"/>
+      <c r="AF7" s="2" t="inlineStr"/>
+      <c r="AG7" s="2" t="inlineStr"/>
+      <c r="AH7" s="2" t="inlineStr"/>
+      <c r="AI7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1549,6 +1609,11 @@
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr"/>
       <c r="AD8" s="2" t="inlineStr"/>
+      <c r="AE8" s="2" t="inlineStr"/>
+      <c r="AF8" s="2" t="inlineStr"/>
+      <c r="AG8" s="2" t="inlineStr"/>
+      <c r="AH8" s="2" t="inlineStr"/>
+      <c r="AI8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1675,6 +1740,11 @@
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr"/>
       <c r="AD9" s="2" t="inlineStr"/>
+      <c r="AE9" s="2" t="inlineStr"/>
+      <c r="AF9" s="2" t="inlineStr"/>
+      <c r="AG9" s="2" t="inlineStr"/>
+      <c r="AH9" s="2" t="inlineStr"/>
+      <c r="AI9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1801,6 +1871,11 @@
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr"/>
       <c r="AD10" s="2" t="inlineStr"/>
+      <c r="AE10" s="2" t="inlineStr"/>
+      <c r="AF10" s="2" t="inlineStr"/>
+      <c r="AG10" s="2" t="inlineStr"/>
+      <c r="AH10" s="2" t="inlineStr"/>
+      <c r="AI10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1927,6 +2002,11 @@
       <c r="AB11" s="2" t="inlineStr"/>
       <c r="AC11" s="2" t="inlineStr"/>
       <c r="AD11" s="2" t="inlineStr"/>
+      <c r="AE11" s="2" t="inlineStr"/>
+      <c r="AF11" s="2" t="inlineStr"/>
+      <c r="AG11" s="2" t="inlineStr"/>
+      <c r="AH11" s="2" t="inlineStr"/>
+      <c r="AI11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2053,6 +2133,11 @@
       <c r="AB12" s="2" t="inlineStr"/>
       <c r="AC12" s="2" t="inlineStr"/>
       <c r="AD12" s="2" t="inlineStr"/>
+      <c r="AE12" s="2" t="inlineStr"/>
+      <c r="AF12" s="2" t="inlineStr"/>
+      <c r="AG12" s="2" t="inlineStr"/>
+      <c r="AH12" s="2" t="inlineStr"/>
+      <c r="AI12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2179,6 +2264,11 @@
       <c r="AB13" s="2" t="inlineStr"/>
       <c r="AC13" s="2" t="inlineStr"/>
       <c r="AD13" s="2" t="inlineStr"/>
+      <c r="AE13" s="2" t="inlineStr"/>
+      <c r="AF13" s="2" t="inlineStr"/>
+      <c r="AG13" s="2" t="inlineStr"/>
+      <c r="AH13" s="2" t="inlineStr"/>
+      <c r="AI13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2305,6 +2395,11 @@
       <c r="AB14" s="2" t="inlineStr"/>
       <c r="AC14" s="2" t="inlineStr"/>
       <c r="AD14" s="2" t="inlineStr"/>
+      <c r="AE14" s="2" t="inlineStr"/>
+      <c r="AF14" s="2" t="inlineStr"/>
+      <c r="AG14" s="2" t="inlineStr"/>
+      <c r="AH14" s="2" t="inlineStr"/>
+      <c r="AI14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2431,6 +2526,11 @@
       <c r="AB15" s="2" t="inlineStr"/>
       <c r="AC15" s="2" t="inlineStr"/>
       <c r="AD15" s="2" t="inlineStr"/>
+      <c r="AE15" s="2" t="inlineStr"/>
+      <c r="AF15" s="2" t="inlineStr"/>
+      <c r="AG15" s="2" t="inlineStr"/>
+      <c r="AH15" s="2" t="inlineStr"/>
+      <c r="AI15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2557,6 +2657,11 @@
       <c r="AB16" s="2" t="inlineStr"/>
       <c r="AC16" s="2" t="inlineStr"/>
       <c r="AD16" s="2" t="inlineStr"/>
+      <c r="AE16" s="2" t="inlineStr"/>
+      <c r="AF16" s="2" t="inlineStr"/>
+      <c r="AG16" s="2" t="inlineStr"/>
+      <c r="AH16" s="2" t="inlineStr"/>
+      <c r="AI16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2683,6 +2788,11 @@
       <c r="AB17" s="2" t="inlineStr"/>
       <c r="AC17" s="2" t="inlineStr"/>
       <c r="AD17" s="2" t="inlineStr"/>
+      <c r="AE17" s="2" t="inlineStr"/>
+      <c r="AF17" s="2" t="inlineStr"/>
+      <c r="AG17" s="2" t="inlineStr"/>
+      <c r="AH17" s="2" t="inlineStr"/>
+      <c r="AI17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2809,6 +2919,11 @@
       <c r="AB18" s="2" t="inlineStr"/>
       <c r="AC18" s="2" t="inlineStr"/>
       <c r="AD18" s="2" t="inlineStr"/>
+      <c r="AE18" s="2" t="inlineStr"/>
+      <c r="AF18" s="2" t="inlineStr"/>
+      <c r="AG18" s="2" t="inlineStr"/>
+      <c r="AH18" s="2" t="inlineStr"/>
+      <c r="AI18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2935,6 +3050,11 @@
       <c r="AB19" s="2" t="inlineStr"/>
       <c r="AC19" s="2" t="inlineStr"/>
       <c r="AD19" s="2" t="inlineStr"/>
+      <c r="AE19" s="2" t="inlineStr"/>
+      <c r="AF19" s="2" t="inlineStr"/>
+      <c r="AG19" s="2" t="inlineStr"/>
+      <c r="AH19" s="2" t="inlineStr"/>
+      <c r="AI19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -3061,6 +3181,11 @@
       <c r="AB20" s="2" t="inlineStr"/>
       <c r="AC20" s="2" t="inlineStr"/>
       <c r="AD20" s="2" t="inlineStr"/>
+      <c r="AE20" s="2" t="inlineStr"/>
+      <c r="AF20" s="2" t="inlineStr"/>
+      <c r="AG20" s="2" t="inlineStr"/>
+      <c r="AH20" s="2" t="inlineStr"/>
+      <c r="AI20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -3187,6 +3312,11 @@
       <c r="AB21" s="2" t="inlineStr"/>
       <c r="AC21" s="2" t="inlineStr"/>
       <c r="AD21" s="2" t="inlineStr"/>
+      <c r="AE21" s="2" t="inlineStr"/>
+      <c r="AF21" s="2" t="inlineStr"/>
+      <c r="AG21" s="2" t="inlineStr"/>
+      <c r="AH21" s="2" t="inlineStr"/>
+      <c r="AI21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -3313,6 +3443,11 @@
       <c r="AB22" s="2" t="inlineStr"/>
       <c r="AC22" s="2" t="inlineStr"/>
       <c r="AD22" s="2" t="inlineStr"/>
+      <c r="AE22" s="2" t="inlineStr"/>
+      <c r="AF22" s="2" t="inlineStr"/>
+      <c r="AG22" s="2" t="inlineStr"/>
+      <c r="AH22" s="2" t="inlineStr"/>
+      <c r="AI22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -3439,6 +3574,11 @@
       <c r="AB23" s="2" t="inlineStr"/>
       <c r="AC23" s="2" t="inlineStr"/>
       <c r="AD23" s="2" t="inlineStr"/>
+      <c r="AE23" s="2" t="inlineStr"/>
+      <c r="AF23" s="2" t="inlineStr"/>
+      <c r="AG23" s="2" t="inlineStr"/>
+      <c r="AH23" s="2" t="inlineStr"/>
+      <c r="AI23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -3565,6 +3705,11 @@
       <c r="AB24" s="2" t="inlineStr"/>
       <c r="AC24" s="2" t="inlineStr"/>
       <c r="AD24" s="2" t="inlineStr"/>
+      <c r="AE24" s="2" t="inlineStr"/>
+      <c r="AF24" s="2" t="inlineStr"/>
+      <c r="AG24" s="2" t="inlineStr"/>
+      <c r="AH24" s="2" t="inlineStr"/>
+      <c r="AI24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -3691,6 +3836,11 @@
       <c r="AB25" s="2" t="inlineStr"/>
       <c r="AC25" s="2" t="inlineStr"/>
       <c r="AD25" s="2" t="inlineStr"/>
+      <c r="AE25" s="2" t="inlineStr"/>
+      <c r="AF25" s="2" t="inlineStr"/>
+      <c r="AG25" s="2" t="inlineStr"/>
+      <c r="AH25" s="2" t="inlineStr"/>
+      <c r="AI25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -3817,6 +3967,11 @@
       <c r="AB26" s="2" t="inlineStr"/>
       <c r="AC26" s="2" t="inlineStr"/>
       <c r="AD26" s="2" t="inlineStr"/>
+      <c r="AE26" s="2" t="inlineStr"/>
+      <c r="AF26" s="2" t="inlineStr"/>
+      <c r="AG26" s="2" t="inlineStr"/>
+      <c r="AH26" s="2" t="inlineStr"/>
+      <c r="AI26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -3943,6 +4098,11 @@
       <c r="AB27" s="2" t="inlineStr"/>
       <c r="AC27" s="2" t="inlineStr"/>
       <c r="AD27" s="2" t="inlineStr"/>
+      <c r="AE27" s="2" t="inlineStr"/>
+      <c r="AF27" s="2" t="inlineStr"/>
+      <c r="AG27" s="2" t="inlineStr"/>
+      <c r="AH27" s="2" t="inlineStr"/>
+      <c r="AI27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -4069,6 +4229,11 @@
       <c r="AB28" s="2" t="inlineStr"/>
       <c r="AC28" s="2" t="inlineStr"/>
       <c r="AD28" s="2" t="inlineStr"/>
+      <c r="AE28" s="2" t="inlineStr"/>
+      <c r="AF28" s="2" t="inlineStr"/>
+      <c r="AG28" s="2" t="inlineStr"/>
+      <c r="AH28" s="2" t="inlineStr"/>
+      <c r="AI28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -4195,6 +4360,11 @@
       <c r="AB29" s="2" t="inlineStr"/>
       <c r="AC29" s="2" t="inlineStr"/>
       <c r="AD29" s="2" t="inlineStr"/>
+      <c r="AE29" s="2" t="inlineStr"/>
+      <c r="AF29" s="2" t="inlineStr"/>
+      <c r="AG29" s="2" t="inlineStr"/>
+      <c r="AH29" s="2" t="inlineStr"/>
+      <c r="AI29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -4321,6 +4491,11 @@
       <c r="AB30" s="2" t="inlineStr"/>
       <c r="AC30" s="2" t="inlineStr"/>
       <c r="AD30" s="2" t="inlineStr"/>
+      <c r="AE30" s="2" t="inlineStr"/>
+      <c r="AF30" s="2" t="inlineStr"/>
+      <c r="AG30" s="2" t="inlineStr"/>
+      <c r="AH30" s="2" t="inlineStr"/>
+      <c r="AI30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -4447,6 +4622,11 @@
       <c r="AB31" s="2" t="inlineStr"/>
       <c r="AC31" s="2" t="inlineStr"/>
       <c r="AD31" s="2" t="inlineStr"/>
+      <c r="AE31" s="2" t="inlineStr"/>
+      <c r="AF31" s="2" t="inlineStr"/>
+      <c r="AG31" s="2" t="inlineStr"/>
+      <c r="AH31" s="2" t="inlineStr"/>
+      <c r="AI31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -4573,6 +4753,11 @@
       <c r="AB32" s="2" t="inlineStr"/>
       <c r="AC32" s="2" t="inlineStr"/>
       <c r="AD32" s="2" t="inlineStr"/>
+      <c r="AE32" s="2" t="inlineStr"/>
+      <c r="AF32" s="2" t="inlineStr"/>
+      <c r="AG32" s="2" t="inlineStr"/>
+      <c r="AH32" s="2" t="inlineStr"/>
+      <c r="AI32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -4699,6 +4884,11 @@
       <c r="AB33" s="2" t="inlineStr"/>
       <c r="AC33" s="2" t="inlineStr"/>
       <c r="AD33" s="2" t="inlineStr"/>
+      <c r="AE33" s="2" t="inlineStr"/>
+      <c r="AF33" s="2" t="inlineStr"/>
+      <c r="AG33" s="2" t="inlineStr"/>
+      <c r="AH33" s="2" t="inlineStr"/>
+      <c r="AI33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -4825,6 +5015,11 @@
       <c r="AB34" s="2" t="inlineStr"/>
       <c r="AC34" s="2" t="inlineStr"/>
       <c r="AD34" s="2" t="inlineStr"/>
+      <c r="AE34" s="2" t="inlineStr"/>
+      <c r="AF34" s="2" t="inlineStr"/>
+      <c r="AG34" s="2" t="inlineStr"/>
+      <c r="AH34" s="2" t="inlineStr"/>
+      <c r="AI34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -4951,6 +5146,11 @@
       <c r="AB35" s="2" t="inlineStr"/>
       <c r="AC35" s="2" t="inlineStr"/>
       <c r="AD35" s="2" t="inlineStr"/>
+      <c r="AE35" s="2" t="inlineStr"/>
+      <c r="AF35" s="2" t="inlineStr"/>
+      <c r="AG35" s="2" t="inlineStr"/>
+      <c r="AH35" s="2" t="inlineStr"/>
+      <c r="AI35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -5077,6 +5277,11 @@
       <c r="AB36" s="2" t="inlineStr"/>
       <c r="AC36" s="2" t="inlineStr"/>
       <c r="AD36" s="2" t="inlineStr"/>
+      <c r="AE36" s="2" t="inlineStr"/>
+      <c r="AF36" s="2" t="inlineStr"/>
+      <c r="AG36" s="2" t="inlineStr"/>
+      <c r="AH36" s="2" t="inlineStr"/>
+      <c r="AI36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -5203,6 +5408,11 @@
       <c r="AB37" s="2" t="inlineStr"/>
       <c r="AC37" s="2" t="inlineStr"/>
       <c r="AD37" s="2" t="inlineStr"/>
+      <c r="AE37" s="2" t="inlineStr"/>
+      <c r="AF37" s="2" t="inlineStr"/>
+      <c r="AG37" s="2" t="inlineStr"/>
+      <c r="AH37" s="2" t="inlineStr"/>
+      <c r="AI37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -5329,6 +5539,11 @@
       <c r="AB38" s="2" t="inlineStr"/>
       <c r="AC38" s="2" t="inlineStr"/>
       <c r="AD38" s="2" t="inlineStr"/>
+      <c r="AE38" s="2" t="inlineStr"/>
+      <c r="AF38" s="2" t="inlineStr"/>
+      <c r="AG38" s="2" t="inlineStr"/>
+      <c r="AH38" s="2" t="inlineStr"/>
+      <c r="AI38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -5455,6 +5670,11 @@
       <c r="AB39" s="2" t="inlineStr"/>
       <c r="AC39" s="2" t="inlineStr"/>
       <c r="AD39" s="2" t="inlineStr"/>
+      <c r="AE39" s="2" t="inlineStr"/>
+      <c r="AF39" s="2" t="inlineStr"/>
+      <c r="AG39" s="2" t="inlineStr"/>
+      <c r="AH39" s="2" t="inlineStr"/>
+      <c r="AI39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -5581,6 +5801,11 @@
       <c r="AB40" s="2" t="inlineStr"/>
       <c r="AC40" s="2" t="inlineStr"/>
       <c r="AD40" s="2" t="inlineStr"/>
+      <c r="AE40" s="2" t="inlineStr"/>
+      <c r="AF40" s="2" t="inlineStr"/>
+      <c r="AG40" s="2" t="inlineStr"/>
+      <c r="AH40" s="2" t="inlineStr"/>
+      <c r="AI40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -5707,6 +5932,11 @@
       <c r="AB41" s="2" t="inlineStr"/>
       <c r="AC41" s="2" t="inlineStr"/>
       <c r="AD41" s="2" t="inlineStr"/>
+      <c r="AE41" s="2" t="inlineStr"/>
+      <c r="AF41" s="2" t="inlineStr"/>
+      <c r="AG41" s="2" t="inlineStr"/>
+      <c r="AH41" s="2" t="inlineStr"/>
+      <c r="AI41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -5833,6 +6063,11 @@
       <c r="AB42" s="2" t="inlineStr"/>
       <c r="AC42" s="2" t="inlineStr"/>
       <c r="AD42" s="2" t="inlineStr"/>
+      <c r="AE42" s="2" t="inlineStr"/>
+      <c r="AF42" s="2" t="inlineStr"/>
+      <c r="AG42" s="2" t="inlineStr"/>
+      <c r="AH42" s="2" t="inlineStr"/>
+      <c r="AI42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -5959,6 +6194,11 @@
       <c r="AB43" s="2" t="inlineStr"/>
       <c r="AC43" s="2" t="inlineStr"/>
       <c r="AD43" s="2" t="inlineStr"/>
+      <c r="AE43" s="2" t="inlineStr"/>
+      <c r="AF43" s="2" t="inlineStr"/>
+      <c r="AG43" s="2" t="inlineStr"/>
+      <c r="AH43" s="2" t="inlineStr"/>
+      <c r="AI43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -6085,6 +6325,11 @@
       <c r="AB44" s="2" t="inlineStr"/>
       <c r="AC44" s="2" t="inlineStr"/>
       <c r="AD44" s="2" t="inlineStr"/>
+      <c r="AE44" s="2" t="inlineStr"/>
+      <c r="AF44" s="2" t="inlineStr"/>
+      <c r="AG44" s="2" t="inlineStr"/>
+      <c r="AH44" s="2" t="inlineStr"/>
+      <c r="AI44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -6211,6 +6456,11 @@
       <c r="AB45" s="2" t="inlineStr"/>
       <c r="AC45" s="2" t="inlineStr"/>
       <c r="AD45" s="2" t="inlineStr"/>
+      <c r="AE45" s="2" t="inlineStr"/>
+      <c r="AF45" s="2" t="inlineStr"/>
+      <c r="AG45" s="2" t="inlineStr"/>
+      <c r="AH45" s="2" t="inlineStr"/>
+      <c r="AI45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -6337,6 +6587,11 @@
       <c r="AB46" s="2" t="inlineStr"/>
       <c r="AC46" s="2" t="inlineStr"/>
       <c r="AD46" s="2" t="inlineStr"/>
+      <c r="AE46" s="2" t="inlineStr"/>
+      <c r="AF46" s="2" t="inlineStr"/>
+      <c r="AG46" s="2" t="inlineStr"/>
+      <c r="AH46" s="2" t="inlineStr"/>
+      <c r="AI46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -6463,6 +6718,11 @@
       <c r="AB47" s="2" t="inlineStr"/>
       <c r="AC47" s="2" t="inlineStr"/>
       <c r="AD47" s="2" t="inlineStr"/>
+      <c r="AE47" s="2" t="inlineStr"/>
+      <c r="AF47" s="2" t="inlineStr"/>
+      <c r="AG47" s="2" t="inlineStr"/>
+      <c r="AH47" s="2" t="inlineStr"/>
+      <c r="AI47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -6589,6 +6849,11 @@
       <c r="AB48" s="2" t="inlineStr"/>
       <c r="AC48" s="2" t="inlineStr"/>
       <c r="AD48" s="2" t="inlineStr"/>
+      <c r="AE48" s="2" t="inlineStr"/>
+      <c r="AF48" s="2" t="inlineStr"/>
+      <c r="AG48" s="2" t="inlineStr"/>
+      <c r="AH48" s="2" t="inlineStr"/>
+      <c r="AI48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -6715,6 +6980,11 @@
       <c r="AB49" s="2" t="inlineStr"/>
       <c r="AC49" s="2" t="inlineStr"/>
       <c r="AD49" s="2" t="inlineStr"/>
+      <c r="AE49" s="2" t="inlineStr"/>
+      <c r="AF49" s="2" t="inlineStr"/>
+      <c r="AG49" s="2" t="inlineStr"/>
+      <c r="AH49" s="2" t="inlineStr"/>
+      <c r="AI49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -6841,6 +7111,11 @@
       <c r="AB50" s="2" t="inlineStr"/>
       <c r="AC50" s="2" t="inlineStr"/>
       <c r="AD50" s="2" t="inlineStr"/>
+      <c r="AE50" s="2" t="inlineStr"/>
+      <c r="AF50" s="2" t="inlineStr"/>
+      <c r="AG50" s="2" t="inlineStr"/>
+      <c r="AH50" s="2" t="inlineStr"/>
+      <c r="AI50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -6967,6 +7242,11 @@
       <c r="AB51" s="2" t="inlineStr"/>
       <c r="AC51" s="2" t="inlineStr"/>
       <c r="AD51" s="2" t="inlineStr"/>
+      <c r="AE51" s="2" t="inlineStr"/>
+      <c r="AF51" s="2" t="inlineStr"/>
+      <c r="AG51" s="2" t="inlineStr"/>
+      <c r="AH51" s="2" t="inlineStr"/>
+      <c r="AI51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -7093,6 +7373,11 @@
       <c r="AB52" s="2" t="inlineStr"/>
       <c r="AC52" s="2" t="inlineStr"/>
       <c r="AD52" s="2" t="inlineStr"/>
+      <c r="AE52" s="2" t="inlineStr"/>
+      <c r="AF52" s="2" t="inlineStr"/>
+      <c r="AG52" s="2" t="inlineStr"/>
+      <c r="AH52" s="2" t="inlineStr"/>
+      <c r="AI52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -7219,6 +7504,11 @@
       <c r="AB53" s="2" t="inlineStr"/>
       <c r="AC53" s="2" t="inlineStr"/>
       <c r="AD53" s="2" t="inlineStr"/>
+      <c r="AE53" s="2" t="inlineStr"/>
+      <c r="AF53" s="2" t="inlineStr"/>
+      <c r="AG53" s="2" t="inlineStr"/>
+      <c r="AH53" s="2" t="inlineStr"/>
+      <c r="AI53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -7345,6 +7635,11 @@
       <c r="AB54" s="2" t="inlineStr"/>
       <c r="AC54" s="2" t="inlineStr"/>
       <c r="AD54" s="2" t="inlineStr"/>
+      <c r="AE54" s="2" t="inlineStr"/>
+      <c r="AF54" s="2" t="inlineStr"/>
+      <c r="AG54" s="2" t="inlineStr"/>
+      <c r="AH54" s="2" t="inlineStr"/>
+      <c r="AI54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -7471,6 +7766,11 @@
       <c r="AB55" s="2" t="inlineStr"/>
       <c r="AC55" s="2" t="inlineStr"/>
       <c r="AD55" s="2" t="inlineStr"/>
+      <c r="AE55" s="2" t="inlineStr"/>
+      <c r="AF55" s="2" t="inlineStr"/>
+      <c r="AG55" s="2" t="inlineStr"/>
+      <c r="AH55" s="2" t="inlineStr"/>
+      <c r="AI55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -7597,6 +7897,11 @@
       <c r="AB56" s="2" t="inlineStr"/>
       <c r="AC56" s="2" t="inlineStr"/>
       <c r="AD56" s="2" t="inlineStr"/>
+      <c r="AE56" s="2" t="inlineStr"/>
+      <c r="AF56" s="2" t="inlineStr"/>
+      <c r="AG56" s="2" t="inlineStr"/>
+      <c r="AH56" s="2" t="inlineStr"/>
+      <c r="AI56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -7723,6 +8028,11 @@
       <c r="AB57" s="2" t="inlineStr"/>
       <c r="AC57" s="2" t="inlineStr"/>
       <c r="AD57" s="2" t="inlineStr"/>
+      <c r="AE57" s="2" t="inlineStr"/>
+      <c r="AF57" s="2" t="inlineStr"/>
+      <c r="AG57" s="2" t="inlineStr"/>
+      <c r="AH57" s="2" t="inlineStr"/>
+      <c r="AI57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -7849,6 +8159,11 @@
       <c r="AB58" s="2" t="inlineStr"/>
       <c r="AC58" s="2" t="inlineStr"/>
       <c r="AD58" s="2" t="inlineStr"/>
+      <c r="AE58" s="2" t="inlineStr"/>
+      <c r="AF58" s="2" t="inlineStr"/>
+      <c r="AG58" s="2" t="inlineStr"/>
+      <c r="AH58" s="2" t="inlineStr"/>
+      <c r="AI58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -7975,6 +8290,11 @@
       <c r="AB59" s="2" t="inlineStr"/>
       <c r="AC59" s="2" t="inlineStr"/>
       <c r="AD59" s="2" t="inlineStr"/>
+      <c r="AE59" s="2" t="inlineStr"/>
+      <c r="AF59" s="2" t="inlineStr"/>
+      <c r="AG59" s="2" t="inlineStr"/>
+      <c r="AH59" s="2" t="inlineStr"/>
+      <c r="AI59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -8101,6 +8421,11 @@
       <c r="AB60" s="2" t="inlineStr"/>
       <c r="AC60" s="2" t="inlineStr"/>
       <c r="AD60" s="2" t="inlineStr"/>
+      <c r="AE60" s="2" t="inlineStr"/>
+      <c r="AF60" s="2" t="inlineStr"/>
+      <c r="AG60" s="2" t="inlineStr"/>
+      <c r="AH60" s="2" t="inlineStr"/>
+      <c r="AI60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -8227,6 +8552,11 @@
       <c r="AB61" s="2" t="inlineStr"/>
       <c r="AC61" s="2" t="inlineStr"/>
       <c r="AD61" s="2" t="inlineStr"/>
+      <c r="AE61" s="2" t="inlineStr"/>
+      <c r="AF61" s="2" t="inlineStr"/>
+      <c r="AG61" s="2" t="inlineStr"/>
+      <c r="AH61" s="2" t="inlineStr"/>
+      <c r="AI61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -8353,6 +8683,11 @@
       <c r="AB62" s="2" t="inlineStr"/>
       <c r="AC62" s="2" t="inlineStr"/>
       <c r="AD62" s="2" t="inlineStr"/>
+      <c r="AE62" s="2" t="inlineStr"/>
+      <c r="AF62" s="2" t="inlineStr"/>
+      <c r="AG62" s="2" t="inlineStr"/>
+      <c r="AH62" s="2" t="inlineStr"/>
+      <c r="AI62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -8479,6 +8814,11 @@
       <c r="AB63" s="2" t="inlineStr"/>
       <c r="AC63" s="2" t="inlineStr"/>
       <c r="AD63" s="2" t="inlineStr"/>
+      <c r="AE63" s="2" t="inlineStr"/>
+      <c r="AF63" s="2" t="inlineStr"/>
+      <c r="AG63" s="2" t="inlineStr"/>
+      <c r="AH63" s="2" t="inlineStr"/>
+      <c r="AI63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -8605,6 +8945,11 @@
       <c r="AB64" s="2" t="inlineStr"/>
       <c r="AC64" s="2" t="inlineStr"/>
       <c r="AD64" s="2" t="inlineStr"/>
+      <c r="AE64" s="2" t="inlineStr"/>
+      <c r="AF64" s="2" t="inlineStr"/>
+      <c r="AG64" s="2" t="inlineStr"/>
+      <c r="AH64" s="2" t="inlineStr"/>
+      <c r="AI64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -8731,6 +9076,11 @@
       <c r="AB65" s="2" t="inlineStr"/>
       <c r="AC65" s="2" t="inlineStr"/>
       <c r="AD65" s="2" t="inlineStr"/>
+      <c r="AE65" s="2" t="inlineStr"/>
+      <c r="AF65" s="2" t="inlineStr"/>
+      <c r="AG65" s="2" t="inlineStr"/>
+      <c r="AH65" s="2" t="inlineStr"/>
+      <c r="AI65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -8857,6 +9207,11 @@
       <c r="AB66" s="2" t="inlineStr"/>
       <c r="AC66" s="2" t="inlineStr"/>
       <c r="AD66" s="2" t="inlineStr"/>
+      <c r="AE66" s="2" t="inlineStr"/>
+      <c r="AF66" s="2" t="inlineStr"/>
+      <c r="AG66" s="2" t="inlineStr"/>
+      <c r="AH66" s="2" t="inlineStr"/>
+      <c r="AI66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -8983,6 +9338,11 @@
       <c r="AB67" s="2" t="inlineStr"/>
       <c r="AC67" s="2" t="inlineStr"/>
       <c r="AD67" s="2" t="inlineStr"/>
+      <c r="AE67" s="2" t="inlineStr"/>
+      <c r="AF67" s="2" t="inlineStr"/>
+      <c r="AG67" s="2" t="inlineStr"/>
+      <c r="AH67" s="2" t="inlineStr"/>
+      <c r="AI67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -9109,6 +9469,11 @@
       <c r="AB68" s="2" t="inlineStr"/>
       <c r="AC68" s="2" t="inlineStr"/>
       <c r="AD68" s="2" t="inlineStr"/>
+      <c r="AE68" s="2" t="inlineStr"/>
+      <c r="AF68" s="2" t="inlineStr"/>
+      <c r="AG68" s="2" t="inlineStr"/>
+      <c r="AH68" s="2" t="inlineStr"/>
+      <c r="AI68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -9235,6 +9600,11 @@
       <c r="AB69" s="2" t="inlineStr"/>
       <c r="AC69" s="2" t="inlineStr"/>
       <c r="AD69" s="2" t="inlineStr"/>
+      <c r="AE69" s="2" t="inlineStr"/>
+      <c r="AF69" s="2" t="inlineStr"/>
+      <c r="AG69" s="2" t="inlineStr"/>
+      <c r="AH69" s="2" t="inlineStr"/>
+      <c r="AI69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -9361,6 +9731,11 @@
       <c r="AB70" s="2" t="inlineStr"/>
       <c r="AC70" s="2" t="inlineStr"/>
       <c r="AD70" s="2" t="inlineStr"/>
+      <c r="AE70" s="2" t="inlineStr"/>
+      <c r="AF70" s="2" t="inlineStr"/>
+      <c r="AG70" s="2" t="inlineStr"/>
+      <c r="AH70" s="2" t="inlineStr"/>
+      <c r="AI70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -9487,6 +9862,11 @@
       <c r="AB71" s="2" t="inlineStr"/>
       <c r="AC71" s="2" t="inlineStr"/>
       <c r="AD71" s="2" t="inlineStr"/>
+      <c r="AE71" s="2" t="inlineStr"/>
+      <c r="AF71" s="2" t="inlineStr"/>
+      <c r="AG71" s="2" t="inlineStr"/>
+      <c r="AH71" s="2" t="inlineStr"/>
+      <c r="AI71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -9613,6 +9993,11 @@
       <c r="AB72" s="2" t="inlineStr"/>
       <c r="AC72" s="2" t="inlineStr"/>
       <c r="AD72" s="2" t="inlineStr"/>
+      <c r="AE72" s="2" t="inlineStr"/>
+      <c r="AF72" s="2" t="inlineStr"/>
+      <c r="AG72" s="2" t="inlineStr"/>
+      <c r="AH72" s="2" t="inlineStr"/>
+      <c r="AI72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -9739,6 +10124,11 @@
       <c r="AB73" s="2" t="inlineStr"/>
       <c r="AC73" s="2" t="inlineStr"/>
       <c r="AD73" s="2" t="inlineStr"/>
+      <c r="AE73" s="2" t="inlineStr"/>
+      <c r="AF73" s="2" t="inlineStr"/>
+      <c r="AG73" s="2" t="inlineStr"/>
+      <c r="AH73" s="2" t="inlineStr"/>
+      <c r="AI73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -9865,6 +10255,11 @@
       <c r="AB74" s="2" t="inlineStr"/>
       <c r="AC74" s="2" t="inlineStr"/>
       <c r="AD74" s="2" t="inlineStr"/>
+      <c r="AE74" s="2" t="inlineStr"/>
+      <c r="AF74" s="2" t="inlineStr"/>
+      <c r="AG74" s="2" t="inlineStr"/>
+      <c r="AH74" s="2" t="inlineStr"/>
+      <c r="AI74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -9991,6 +10386,11 @@
       <c r="AB75" s="2" t="inlineStr"/>
       <c r="AC75" s="2" t="inlineStr"/>
       <c r="AD75" s="2" t="inlineStr"/>
+      <c r="AE75" s="2" t="inlineStr"/>
+      <c r="AF75" s="2" t="inlineStr"/>
+      <c r="AG75" s="2" t="inlineStr"/>
+      <c r="AH75" s="2" t="inlineStr"/>
+      <c r="AI75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -10117,6 +10517,11 @@
       <c r="AB76" s="2" t="inlineStr"/>
       <c r="AC76" s="2" t="inlineStr"/>
       <c r="AD76" s="2" t="inlineStr"/>
+      <c r="AE76" s="2" t="inlineStr"/>
+      <c r="AF76" s="2" t="inlineStr"/>
+      <c r="AG76" s="2" t="inlineStr"/>
+      <c r="AH76" s="2" t="inlineStr"/>
+      <c r="AI76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -10243,6 +10648,11 @@
       <c r="AB77" s="2" t="inlineStr"/>
       <c r="AC77" s="2" t="inlineStr"/>
       <c r="AD77" s="2" t="inlineStr"/>
+      <c r="AE77" s="2" t="inlineStr"/>
+      <c r="AF77" s="2" t="inlineStr"/>
+      <c r="AG77" s="2" t="inlineStr"/>
+      <c r="AH77" s="2" t="inlineStr"/>
+      <c r="AI77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -10369,6 +10779,11 @@
       <c r="AB78" s="2" t="inlineStr"/>
       <c r="AC78" s="2" t="inlineStr"/>
       <c r="AD78" s="2" t="inlineStr"/>
+      <c r="AE78" s="2" t="inlineStr"/>
+      <c r="AF78" s="2" t="inlineStr"/>
+      <c r="AG78" s="2" t="inlineStr"/>
+      <c r="AH78" s="2" t="inlineStr"/>
+      <c r="AI78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -10495,6 +10910,11 @@
       <c r="AB79" s="2" t="inlineStr"/>
       <c r="AC79" s="2" t="inlineStr"/>
       <c r="AD79" s="2" t="inlineStr"/>
+      <c r="AE79" s="2" t="inlineStr"/>
+      <c r="AF79" s="2" t="inlineStr"/>
+      <c r="AG79" s="2" t="inlineStr"/>
+      <c r="AH79" s="2" t="inlineStr"/>
+      <c r="AI79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -10621,6 +11041,11 @@
       <c r="AB80" s="2" t="inlineStr"/>
       <c r="AC80" s="2" t="inlineStr"/>
       <c r="AD80" s="2" t="inlineStr"/>
+      <c r="AE80" s="2" t="inlineStr"/>
+      <c r="AF80" s="2" t="inlineStr"/>
+      <c r="AG80" s="2" t="inlineStr"/>
+      <c r="AH80" s="2" t="inlineStr"/>
+      <c r="AI80" s="2" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -10747,6 +11172,11 @@
       <c r="AB81" s="2" t="inlineStr"/>
       <c r="AC81" s="2" t="inlineStr"/>
       <c r="AD81" s="2" t="inlineStr"/>
+      <c r="AE81" s="2" t="inlineStr"/>
+      <c r="AF81" s="2" t="inlineStr"/>
+      <c r="AG81" s="2" t="inlineStr"/>
+      <c r="AH81" s="2" t="inlineStr"/>
+      <c r="AI81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -10873,6 +11303,11 @@
       <c r="AB82" s="2" t="inlineStr"/>
       <c r="AC82" s="2" t="inlineStr"/>
       <c r="AD82" s="2" t="inlineStr"/>
+      <c r="AE82" s="2" t="inlineStr"/>
+      <c r="AF82" s="2" t="inlineStr"/>
+      <c r="AG82" s="2" t="inlineStr"/>
+      <c r="AH82" s="2" t="inlineStr"/>
+      <c r="AI82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -10999,6 +11434,11 @@
       <c r="AB83" s="2" t="inlineStr"/>
       <c r="AC83" s="2" t="inlineStr"/>
       <c r="AD83" s="2" t="inlineStr"/>
+      <c r="AE83" s="2" t="inlineStr"/>
+      <c r="AF83" s="2" t="inlineStr"/>
+      <c r="AG83" s="2" t="inlineStr"/>
+      <c r="AH83" s="2" t="inlineStr"/>
+      <c r="AI83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -11125,6 +11565,11 @@
       <c r="AB84" s="2" t="inlineStr"/>
       <c r="AC84" s="2" t="inlineStr"/>
       <c r="AD84" s="2" t="inlineStr"/>
+      <c r="AE84" s="2" t="inlineStr"/>
+      <c r="AF84" s="2" t="inlineStr"/>
+      <c r="AG84" s="2" t="inlineStr"/>
+      <c r="AH84" s="2" t="inlineStr"/>
+      <c r="AI84" s="2" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -11251,6 +11696,11 @@
       <c r="AB85" s="2" t="inlineStr"/>
       <c r="AC85" s="2" t="inlineStr"/>
       <c r="AD85" s="2" t="inlineStr"/>
+      <c r="AE85" s="2" t="inlineStr"/>
+      <c r="AF85" s="2" t="inlineStr"/>
+      <c r="AG85" s="2" t="inlineStr"/>
+      <c r="AH85" s="2" t="inlineStr"/>
+      <c r="AI85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -11377,6 +11827,11 @@
       <c r="AB86" s="2" t="inlineStr"/>
       <c r="AC86" s="2" t="inlineStr"/>
       <c r="AD86" s="2" t="inlineStr"/>
+      <c r="AE86" s="2" t="inlineStr"/>
+      <c r="AF86" s="2" t="inlineStr"/>
+      <c r="AG86" s="2" t="inlineStr"/>
+      <c r="AH86" s="2" t="inlineStr"/>
+      <c r="AI86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -11503,6 +11958,11 @@
       <c r="AB87" s="2" t="inlineStr"/>
       <c r="AC87" s="2" t="inlineStr"/>
       <c r="AD87" s="2" t="inlineStr"/>
+      <c r="AE87" s="2" t="inlineStr"/>
+      <c r="AF87" s="2" t="inlineStr"/>
+      <c r="AG87" s="2" t="inlineStr"/>
+      <c r="AH87" s="2" t="inlineStr"/>
+      <c r="AI87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -11629,6 +12089,11 @@
       <c r="AB88" s="2" t="inlineStr"/>
       <c r="AC88" s="2" t="inlineStr"/>
       <c r="AD88" s="2" t="inlineStr"/>
+      <c r="AE88" s="2" t="inlineStr"/>
+      <c r="AF88" s="2" t="inlineStr"/>
+      <c r="AG88" s="2" t="inlineStr"/>
+      <c r="AH88" s="2" t="inlineStr"/>
+      <c r="AI88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -11755,6 +12220,11 @@
       <c r="AB89" s="2" t="inlineStr"/>
       <c r="AC89" s="2" t="inlineStr"/>
       <c r="AD89" s="2" t="inlineStr"/>
+      <c r="AE89" s="2" t="inlineStr"/>
+      <c r="AF89" s="2" t="inlineStr"/>
+      <c r="AG89" s="2" t="inlineStr"/>
+      <c r="AH89" s="2" t="inlineStr"/>
+      <c r="AI89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -11881,6 +12351,11 @@
       <c r="AB90" s="2" t="inlineStr"/>
       <c r="AC90" s="2" t="inlineStr"/>
       <c r="AD90" s="2" t="inlineStr"/>
+      <c r="AE90" s="2" t="inlineStr"/>
+      <c r="AF90" s="2" t="inlineStr"/>
+      <c r="AG90" s="2" t="inlineStr"/>
+      <c r="AH90" s="2" t="inlineStr"/>
+      <c r="AI90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -12007,6 +12482,11 @@
       <c r="AB91" s="2" t="inlineStr"/>
       <c r="AC91" s="2" t="inlineStr"/>
       <c r="AD91" s="2" t="inlineStr"/>
+      <c r="AE91" s="2" t="inlineStr"/>
+      <c r="AF91" s="2" t="inlineStr"/>
+      <c r="AG91" s="2" t="inlineStr"/>
+      <c r="AH91" s="2" t="inlineStr"/>
+      <c r="AI91" s="2" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -12133,6 +12613,11 @@
       <c r="AB92" s="2" t="inlineStr"/>
       <c r="AC92" s="2" t="inlineStr"/>
       <c r="AD92" s="2" t="inlineStr"/>
+      <c r="AE92" s="2" t="inlineStr"/>
+      <c r="AF92" s="2" t="inlineStr"/>
+      <c r="AG92" s="2" t="inlineStr"/>
+      <c r="AH92" s="2" t="inlineStr"/>
+      <c r="AI92" s="2" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -12259,6 +12744,11 @@
       <c r="AB93" s="2" t="inlineStr"/>
       <c r="AC93" s="2" t="inlineStr"/>
       <c r="AD93" s="2" t="inlineStr"/>
+      <c r="AE93" s="2" t="inlineStr"/>
+      <c r="AF93" s="2" t="inlineStr"/>
+      <c r="AG93" s="2" t="inlineStr"/>
+      <c r="AH93" s="2" t="inlineStr"/>
+      <c r="AI93" s="2" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -12385,6 +12875,11 @@
       <c r="AB94" s="2" t="inlineStr"/>
       <c r="AC94" s="2" t="inlineStr"/>
       <c r="AD94" s="2" t="inlineStr"/>
+      <c r="AE94" s="2" t="inlineStr"/>
+      <c r="AF94" s="2" t="inlineStr"/>
+      <c r="AG94" s="2" t="inlineStr"/>
+      <c r="AH94" s="2" t="inlineStr"/>
+      <c r="AI94" s="2" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -12511,6 +13006,11 @@
       <c r="AB95" s="2" t="inlineStr"/>
       <c r="AC95" s="2" t="inlineStr"/>
       <c r="AD95" s="2" t="inlineStr"/>
+      <c r="AE95" s="2" t="inlineStr"/>
+      <c r="AF95" s="2" t="inlineStr"/>
+      <c r="AG95" s="2" t="inlineStr"/>
+      <c r="AH95" s="2" t="inlineStr"/>
+      <c r="AI95" s="2" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -12637,6 +13137,11 @@
       <c r="AB96" s="2" t="inlineStr"/>
       <c r="AC96" s="2" t="inlineStr"/>
       <c r="AD96" s="2" t="inlineStr"/>
+      <c r="AE96" s="2" t="inlineStr"/>
+      <c r="AF96" s="2" t="inlineStr"/>
+      <c r="AG96" s="2" t="inlineStr"/>
+      <c r="AH96" s="2" t="inlineStr"/>
+      <c r="AI96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -12763,6 +13268,11 @@
       <c r="AB97" s="2" t="inlineStr"/>
       <c r="AC97" s="2" t="inlineStr"/>
       <c r="AD97" s="2" t="inlineStr"/>
+      <c r="AE97" s="2" t="inlineStr"/>
+      <c r="AF97" s="2" t="inlineStr"/>
+      <c r="AG97" s="2" t="inlineStr"/>
+      <c r="AH97" s="2" t="inlineStr"/>
+      <c r="AI97" s="2" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -12889,6 +13399,11 @@
       <c r="AB98" s="2" t="inlineStr"/>
       <c r="AC98" s="2" t="inlineStr"/>
       <c r="AD98" s="2" t="inlineStr"/>
+      <c r="AE98" s="2" t="inlineStr"/>
+      <c r="AF98" s="2" t="inlineStr"/>
+      <c r="AG98" s="2" t="inlineStr"/>
+      <c r="AH98" s="2" t="inlineStr"/>
+      <c r="AI98" s="2" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -13015,6 +13530,11 @@
       <c r="AB99" s="2" t="inlineStr"/>
       <c r="AC99" s="2" t="inlineStr"/>
       <c r="AD99" s="2" t="inlineStr"/>
+      <c r="AE99" s="2" t="inlineStr"/>
+      <c r="AF99" s="2" t="inlineStr"/>
+      <c r="AG99" s="2" t="inlineStr"/>
+      <c r="AH99" s="2" t="inlineStr"/>
+      <c r="AI99" s="2" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -13141,6 +13661,11 @@
       <c r="AB100" s="2" t="inlineStr"/>
       <c r="AC100" s="2" t="inlineStr"/>
       <c r="AD100" s="2" t="inlineStr"/>
+      <c r="AE100" s="2" t="inlineStr"/>
+      <c r="AF100" s="2" t="inlineStr"/>
+      <c r="AG100" s="2" t="inlineStr"/>
+      <c r="AH100" s="2" t="inlineStr"/>
+      <c r="AI100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -13267,6 +13792,11 @@
       <c r="AB101" s="2" t="inlineStr"/>
       <c r="AC101" s="2" t="inlineStr"/>
       <c r="AD101" s="2" t="inlineStr"/>
+      <c r="AE101" s="2" t="inlineStr"/>
+      <c r="AF101" s="2" t="inlineStr"/>
+      <c r="AG101" s="2" t="inlineStr"/>
+      <c r="AH101" s="2" t="inlineStr"/>
+      <c r="AI101" s="2" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -13393,6 +13923,11 @@
       <c r="AB102" s="2" t="inlineStr"/>
       <c r="AC102" s="2" t="inlineStr"/>
       <c r="AD102" s="2" t="inlineStr"/>
+      <c r="AE102" s="2" t="inlineStr"/>
+      <c r="AF102" s="2" t="inlineStr"/>
+      <c r="AG102" s="2" t="inlineStr"/>
+      <c r="AH102" s="2" t="inlineStr"/>
+      <c r="AI102" s="2" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -13519,6 +14054,11 @@
       <c r="AB103" s="2" t="inlineStr"/>
       <c r="AC103" s="2" t="inlineStr"/>
       <c r="AD103" s="2" t="inlineStr"/>
+      <c r="AE103" s="2" t="inlineStr"/>
+      <c r="AF103" s="2" t="inlineStr"/>
+      <c r="AG103" s="2" t="inlineStr"/>
+      <c r="AH103" s="2" t="inlineStr"/>
+      <c r="AI103" s="2" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -13645,6 +14185,11 @@
       <c r="AB104" s="2" t="inlineStr"/>
       <c r="AC104" s="2" t="inlineStr"/>
       <c r="AD104" s="2" t="inlineStr"/>
+      <c r="AE104" s="2" t="inlineStr"/>
+      <c r="AF104" s="2" t="inlineStr"/>
+      <c r="AG104" s="2" t="inlineStr"/>
+      <c r="AH104" s="2" t="inlineStr"/>
+      <c r="AI104" s="2" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -13771,6 +14316,11 @@
       <c r="AB105" s="2" t="inlineStr"/>
       <c r="AC105" s="2" t="inlineStr"/>
       <c r="AD105" s="2" t="inlineStr"/>
+      <c r="AE105" s="2" t="inlineStr"/>
+      <c r="AF105" s="2" t="inlineStr"/>
+      <c r="AG105" s="2" t="inlineStr"/>
+      <c r="AH105" s="2" t="inlineStr"/>
+      <c r="AI105" s="2" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -13897,6 +14447,11 @@
       <c r="AB106" s="2" t="inlineStr"/>
       <c r="AC106" s="2" t="inlineStr"/>
       <c r="AD106" s="2" t="inlineStr"/>
+      <c r="AE106" s="2" t="inlineStr"/>
+      <c r="AF106" s="2" t="inlineStr"/>
+      <c r="AG106" s="2" t="inlineStr"/>
+      <c r="AH106" s="2" t="inlineStr"/>
+      <c r="AI106" s="2" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -14023,6 +14578,11 @@
       <c r="AB107" s="2" t="inlineStr"/>
       <c r="AC107" s="2" t="inlineStr"/>
       <c r="AD107" s="2" t="inlineStr"/>
+      <c r="AE107" s="2" t="inlineStr"/>
+      <c r="AF107" s="2" t="inlineStr"/>
+      <c r="AG107" s="2" t="inlineStr"/>
+      <c r="AH107" s="2" t="inlineStr"/>
+      <c r="AI107" s="2" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
@@ -14123,6 +14683,11 @@
       <c r="AB108" s="3" t="inlineStr"/>
       <c r="AC108" s="3" t="inlineStr"/>
       <c r="AD108" s="3" t="inlineStr"/>
+      <c r="AE108" s="3" t="inlineStr"/>
+      <c r="AF108" s="3" t="inlineStr"/>
+      <c r="AG108" s="3" t="inlineStr"/>
+      <c r="AH108" s="3" t="inlineStr"/>
+      <c r="AI108" s="3" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -14249,6 +14814,11 @@
       <c r="AB109" s="2" t="inlineStr"/>
       <c r="AC109" s="2" t="inlineStr"/>
       <c r="AD109" s="2" t="inlineStr"/>
+      <c r="AE109" s="2" t="inlineStr"/>
+      <c r="AF109" s="2" t="inlineStr"/>
+      <c r="AG109" s="2" t="inlineStr"/>
+      <c r="AH109" s="2" t="inlineStr"/>
+      <c r="AI109" s="2" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -14375,6 +14945,11 @@
       <c r="AB110" s="2" t="inlineStr"/>
       <c r="AC110" s="2" t="inlineStr"/>
       <c r="AD110" s="2" t="inlineStr"/>
+      <c r="AE110" s="2" t="inlineStr"/>
+      <c r="AF110" s="2" t="inlineStr"/>
+      <c r="AG110" s="2" t="inlineStr"/>
+      <c r="AH110" s="2" t="inlineStr"/>
+      <c r="AI110" s="2" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
@@ -14475,6 +15050,11 @@
       <c r="AB111" s="3" t="inlineStr"/>
       <c r="AC111" s="3" t="inlineStr"/>
       <c r="AD111" s="3" t="inlineStr"/>
+      <c r="AE111" s="3" t="inlineStr"/>
+      <c r="AF111" s="3" t="inlineStr"/>
+      <c r="AG111" s="3" t="inlineStr"/>
+      <c r="AH111" s="3" t="inlineStr"/>
+      <c r="AI111" s="3" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -14601,6 +15181,11 @@
       <c r="AB112" s="2" t="inlineStr"/>
       <c r="AC112" s="2" t="inlineStr"/>
       <c r="AD112" s="2" t="inlineStr"/>
+      <c r="AE112" s="2" t="inlineStr"/>
+      <c r="AF112" s="2" t="inlineStr"/>
+      <c r="AG112" s="2" t="inlineStr"/>
+      <c r="AH112" s="2" t="inlineStr"/>
+      <c r="AI112" s="2" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -14727,6 +15312,11 @@
       <c r="AB113" s="2" t="inlineStr"/>
       <c r="AC113" s="2" t="inlineStr"/>
       <c r="AD113" s="2" t="inlineStr"/>
+      <c r="AE113" s="2" t="inlineStr"/>
+      <c r="AF113" s="2" t="inlineStr"/>
+      <c r="AG113" s="2" t="inlineStr"/>
+      <c r="AH113" s="2" t="inlineStr"/>
+      <c r="AI113" s="2" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -14853,6 +15443,11 @@
       <c r="AB114" s="2" t="inlineStr"/>
       <c r="AC114" s="2" t="inlineStr"/>
       <c r="AD114" s="2" t="inlineStr"/>
+      <c r="AE114" s="2" t="inlineStr"/>
+      <c r="AF114" s="2" t="inlineStr"/>
+      <c r="AG114" s="2" t="inlineStr"/>
+      <c r="AH114" s="2" t="inlineStr"/>
+      <c r="AI114" s="2" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
@@ -14953,6 +15548,11 @@
       <c r="AB115" s="3" t="inlineStr"/>
       <c r="AC115" s="3" t="inlineStr"/>
       <c r="AD115" s="3" t="inlineStr"/>
+      <c r="AE115" s="3" t="inlineStr"/>
+      <c r="AF115" s="3" t="inlineStr"/>
+      <c r="AG115" s="3" t="inlineStr"/>
+      <c r="AH115" s="3" t="inlineStr"/>
+      <c r="AI115" s="3" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -15079,6 +15679,11 @@
       <c r="AB116" s="2" t="inlineStr"/>
       <c r="AC116" s="2" t="inlineStr"/>
       <c r="AD116" s="2" t="inlineStr"/>
+      <c r="AE116" s="2" t="inlineStr"/>
+      <c r="AF116" s="2" t="inlineStr"/>
+      <c r="AG116" s="2" t="inlineStr"/>
+      <c r="AH116" s="2" t="inlineStr"/>
+      <c r="AI116" s="2" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -15205,6 +15810,11 @@
       <c r="AB117" s="2" t="inlineStr"/>
       <c r="AC117" s="2" t="inlineStr"/>
       <c r="AD117" s="2" t="inlineStr"/>
+      <c r="AE117" s="2" t="inlineStr"/>
+      <c r="AF117" s="2" t="inlineStr"/>
+      <c r="AG117" s="2" t="inlineStr"/>
+      <c r="AH117" s="2" t="inlineStr"/>
+      <c r="AI117" s="2" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -15331,6 +15941,11 @@
       <c r="AB118" s="2" t="inlineStr"/>
       <c r="AC118" s="2" t="inlineStr"/>
       <c r="AD118" s="2" t="inlineStr"/>
+      <c r="AE118" s="2" t="inlineStr"/>
+      <c r="AF118" s="2" t="inlineStr"/>
+      <c r="AG118" s="2" t="inlineStr"/>
+      <c r="AH118" s="2" t="inlineStr"/>
+      <c r="AI118" s="2" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -15457,6 +16072,11 @@
       <c r="AB119" s="2" t="inlineStr"/>
       <c r="AC119" s="2" t="inlineStr"/>
       <c r="AD119" s="2" t="inlineStr"/>
+      <c r="AE119" s="2" t="inlineStr"/>
+      <c r="AF119" s="2" t="inlineStr"/>
+      <c r="AG119" s="2" t="inlineStr"/>
+      <c r="AH119" s="2" t="inlineStr"/>
+      <c r="AI119" s="2" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -15583,6 +16203,11 @@
       <c r="AB120" s="2" t="inlineStr"/>
       <c r="AC120" s="2" t="inlineStr"/>
       <c r="AD120" s="2" t="inlineStr"/>
+      <c r="AE120" s="2" t="inlineStr"/>
+      <c r="AF120" s="2" t="inlineStr"/>
+      <c r="AG120" s="2" t="inlineStr"/>
+      <c r="AH120" s="2" t="inlineStr"/>
+      <c r="AI120" s="2" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -15709,6 +16334,11 @@
       <c r="AB121" s="2" t="inlineStr"/>
       <c r="AC121" s="2" t="inlineStr"/>
       <c r="AD121" s="2" t="inlineStr"/>
+      <c r="AE121" s="2" t="inlineStr"/>
+      <c r="AF121" s="2" t="inlineStr"/>
+      <c r="AG121" s="2" t="inlineStr"/>
+      <c r="AH121" s="2" t="inlineStr"/>
+      <c r="AI121" s="2" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -15835,6 +16465,11 @@
       <c r="AB122" s="2" t="inlineStr"/>
       <c r="AC122" s="2" t="inlineStr"/>
       <c r="AD122" s="2" t="inlineStr"/>
+      <c r="AE122" s="2" t="inlineStr"/>
+      <c r="AF122" s="2" t="inlineStr"/>
+      <c r="AG122" s="2" t="inlineStr"/>
+      <c r="AH122" s="2" t="inlineStr"/>
+      <c r="AI122" s="2" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -15961,6 +16596,11 @@
       <c r="AB123" s="2" t="inlineStr"/>
       <c r="AC123" s="2" t="inlineStr"/>
       <c r="AD123" s="2" t="inlineStr"/>
+      <c r="AE123" s="2" t="inlineStr"/>
+      <c r="AF123" s="2" t="inlineStr"/>
+      <c r="AG123" s="2" t="inlineStr"/>
+      <c r="AH123" s="2" t="inlineStr"/>
+      <c r="AI123" s="2" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -16087,6 +16727,11 @@
       <c r="AB124" s="2" t="inlineStr"/>
       <c r="AC124" s="2" t="inlineStr"/>
       <c r="AD124" s="2" t="inlineStr"/>
+      <c r="AE124" s="2" t="inlineStr"/>
+      <c r="AF124" s="2" t="inlineStr"/>
+      <c r="AG124" s="2" t="inlineStr"/>
+      <c r="AH124" s="2" t="inlineStr"/>
+      <c r="AI124" s="2" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -16213,6 +16858,11 @@
       <c r="AB125" s="2" t="inlineStr"/>
       <c r="AC125" s="2" t="inlineStr"/>
       <c r="AD125" s="2" t="inlineStr"/>
+      <c r="AE125" s="2" t="inlineStr"/>
+      <c r="AF125" s="2" t="inlineStr"/>
+      <c r="AG125" s="2" t="inlineStr"/>
+      <c r="AH125" s="2" t="inlineStr"/>
+      <c r="AI125" s="2" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
@@ -16313,6 +16963,11 @@
       <c r="AB126" s="3" t="inlineStr"/>
       <c r="AC126" s="3" t="inlineStr"/>
       <c r="AD126" s="3" t="inlineStr"/>
+      <c r="AE126" s="3" t="inlineStr"/>
+      <c r="AF126" s="3" t="inlineStr"/>
+      <c r="AG126" s="3" t="inlineStr"/>
+      <c r="AH126" s="3" t="inlineStr"/>
+      <c r="AI126" s="3" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -16439,6 +17094,11 @@
       <c r="AB127" s="2" t="inlineStr"/>
       <c r="AC127" s="2" t="inlineStr"/>
       <c r="AD127" s="2" t="inlineStr"/>
+      <c r="AE127" s="2" t="inlineStr"/>
+      <c r="AF127" s="2" t="inlineStr"/>
+      <c r="AG127" s="2" t="inlineStr"/>
+      <c r="AH127" s="2" t="inlineStr"/>
+      <c r="AI127" s="2" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -16565,6 +17225,11 @@
       <c r="AB128" s="2" t="inlineStr"/>
       <c r="AC128" s="2" t="inlineStr"/>
       <c r="AD128" s="2" t="inlineStr"/>
+      <c r="AE128" s="2" t="inlineStr"/>
+      <c r="AF128" s="2" t="inlineStr"/>
+      <c r="AG128" s="2" t="inlineStr"/>
+      <c r="AH128" s="2" t="inlineStr"/>
+      <c r="AI128" s="2" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -16691,6 +17356,11 @@
       <c r="AB129" s="2" t="inlineStr"/>
       <c r="AC129" s="2" t="inlineStr"/>
       <c r="AD129" s="2" t="inlineStr"/>
+      <c r="AE129" s="2" t="inlineStr"/>
+      <c r="AF129" s="2" t="inlineStr"/>
+      <c r="AG129" s="2" t="inlineStr"/>
+      <c r="AH129" s="2" t="inlineStr"/>
+      <c r="AI129" s="2" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -16817,6 +17487,11 @@
       <c r="AB130" s="2" t="inlineStr"/>
       <c r="AC130" s="2" t="inlineStr"/>
       <c r="AD130" s="2" t="inlineStr"/>
+      <c r="AE130" s="2" t="inlineStr"/>
+      <c r="AF130" s="2" t="inlineStr"/>
+      <c r="AG130" s="2" t="inlineStr"/>
+      <c r="AH130" s="2" t="inlineStr"/>
+      <c r="AI130" s="2" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -16943,6 +17618,11 @@
       <c r="AB131" s="2" t="inlineStr"/>
       <c r="AC131" s="2" t="inlineStr"/>
       <c r="AD131" s="2" t="inlineStr"/>
+      <c r="AE131" s="2" t="inlineStr"/>
+      <c r="AF131" s="2" t="inlineStr"/>
+      <c r="AG131" s="2" t="inlineStr"/>
+      <c r="AH131" s="2" t="inlineStr"/>
+      <c r="AI131" s="2" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -17069,6 +17749,11 @@
       <c r="AB132" s="2" t="inlineStr"/>
       <c r="AC132" s="2" t="inlineStr"/>
       <c r="AD132" s="2" t="inlineStr"/>
+      <c r="AE132" s="2" t="inlineStr"/>
+      <c r="AF132" s="2" t="inlineStr"/>
+      <c r="AG132" s="2" t="inlineStr"/>
+      <c r="AH132" s="2" t="inlineStr"/>
+      <c r="AI132" s="2" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -17195,6 +17880,11 @@
       <c r="AB133" s="2" t="inlineStr"/>
       <c r="AC133" s="2" t="inlineStr"/>
       <c r="AD133" s="2" t="inlineStr"/>
+      <c r="AE133" s="2" t="inlineStr"/>
+      <c r="AF133" s="2" t="inlineStr"/>
+      <c r="AG133" s="2" t="inlineStr"/>
+      <c r="AH133" s="2" t="inlineStr"/>
+      <c r="AI133" s="2" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -17321,6 +18011,11 @@
       <c r="AB134" s="2" t="inlineStr"/>
       <c r="AC134" s="2" t="inlineStr"/>
       <c r="AD134" s="2" t="inlineStr"/>
+      <c r="AE134" s="2" t="inlineStr"/>
+      <c r="AF134" s="2" t="inlineStr"/>
+      <c r="AG134" s="2" t="inlineStr"/>
+      <c r="AH134" s="2" t="inlineStr"/>
+      <c r="AI134" s="2" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -17447,6 +18142,11 @@
       <c r="AB135" s="2" t="inlineStr"/>
       <c r="AC135" s="2" t="inlineStr"/>
       <c r="AD135" s="2" t="inlineStr"/>
+      <c r="AE135" s="2" t="inlineStr"/>
+      <c r="AF135" s="2" t="inlineStr"/>
+      <c r="AG135" s="2" t="inlineStr"/>
+      <c r="AH135" s="2" t="inlineStr"/>
+      <c r="AI135" s="2" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -17573,6 +18273,11 @@
       <c r="AB136" s="2" t="inlineStr"/>
       <c r="AC136" s="2" t="inlineStr"/>
       <c r="AD136" s="2" t="inlineStr"/>
+      <c r="AE136" s="2" t="inlineStr"/>
+      <c r="AF136" s="2" t="inlineStr"/>
+      <c r="AG136" s="2" t="inlineStr"/>
+      <c r="AH136" s="2" t="inlineStr"/>
+      <c r="AI136" s="2" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -17699,6 +18404,11 @@
       <c r="AB137" s="2" t="inlineStr"/>
       <c r="AC137" s="2" t="inlineStr"/>
       <c r="AD137" s="2" t="inlineStr"/>
+      <c r="AE137" s="2" t="inlineStr"/>
+      <c r="AF137" s="2" t="inlineStr"/>
+      <c r="AG137" s="2" t="inlineStr"/>
+      <c r="AH137" s="2" t="inlineStr"/>
+      <c r="AI137" s="2" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -17825,6 +18535,11 @@
       <c r="AB138" s="2" t="inlineStr"/>
       <c r="AC138" s="2" t="inlineStr"/>
       <c r="AD138" s="2" t="inlineStr"/>
+      <c r="AE138" s="2" t="inlineStr"/>
+      <c r="AF138" s="2" t="inlineStr"/>
+      <c r="AG138" s="2" t="inlineStr"/>
+      <c r="AH138" s="2" t="inlineStr"/>
+      <c r="AI138" s="2" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -17951,6 +18666,11 @@
       <c r="AB139" s="2" t="inlineStr"/>
       <c r="AC139" s="2" t="inlineStr"/>
       <c r="AD139" s="2" t="inlineStr"/>
+      <c r="AE139" s="2" t="inlineStr"/>
+      <c r="AF139" s="2" t="inlineStr"/>
+      <c r="AG139" s="2" t="inlineStr"/>
+      <c r="AH139" s="2" t="inlineStr"/>
+      <c r="AI139" s="2" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -18077,6 +18797,11 @@
       <c r="AB140" s="2" t="inlineStr"/>
       <c r="AC140" s="2" t="inlineStr"/>
       <c r="AD140" s="2" t="inlineStr"/>
+      <c r="AE140" s="2" t="inlineStr"/>
+      <c r="AF140" s="2" t="inlineStr"/>
+      <c r="AG140" s="2" t="inlineStr"/>
+      <c r="AH140" s="2" t="inlineStr"/>
+      <c r="AI140" s="2" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -18203,6 +18928,11 @@
       <c r="AB141" s="2" t="inlineStr"/>
       <c r="AC141" s="2" t="inlineStr"/>
       <c r="AD141" s="2" t="inlineStr"/>
+      <c r="AE141" s="2" t="inlineStr"/>
+      <c r="AF141" s="2" t="inlineStr"/>
+      <c r="AG141" s="2" t="inlineStr"/>
+      <c r="AH141" s="2" t="inlineStr"/>
+      <c r="AI141" s="2" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -18329,6 +19059,11 @@
       <c r="AB142" s="2" t="inlineStr"/>
       <c r="AC142" s="2" t="inlineStr"/>
       <c r="AD142" s="2" t="inlineStr"/>
+      <c r="AE142" s="2" t="inlineStr"/>
+      <c r="AF142" s="2" t="inlineStr"/>
+      <c r="AG142" s="2" t="inlineStr"/>
+      <c r="AH142" s="2" t="inlineStr"/>
+      <c r="AI142" s="2" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -18455,6 +19190,11 @@
       <c r="AB143" s="2" t="inlineStr"/>
       <c r="AC143" s="2" t="inlineStr"/>
       <c r="AD143" s="2" t="inlineStr"/>
+      <c r="AE143" s="2" t="inlineStr"/>
+      <c r="AF143" s="2" t="inlineStr"/>
+      <c r="AG143" s="2" t="inlineStr"/>
+      <c r="AH143" s="2" t="inlineStr"/>
+      <c r="AI143" s="2" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -18581,6 +19321,11 @@
       <c r="AB144" s="2" t="inlineStr"/>
       <c r="AC144" s="2" t="inlineStr"/>
       <c r="AD144" s="2" t="inlineStr"/>
+      <c r="AE144" s="2" t="inlineStr"/>
+      <c r="AF144" s="2" t="inlineStr"/>
+      <c r="AG144" s="2" t="inlineStr"/>
+      <c r="AH144" s="2" t="inlineStr"/>
+      <c r="AI144" s="2" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -18707,6 +19452,11 @@
       <c r="AB145" s="2" t="inlineStr"/>
       <c r="AC145" s="2" t="inlineStr"/>
       <c r="AD145" s="2" t="inlineStr"/>
+      <c r="AE145" s="2" t="inlineStr"/>
+      <c r="AF145" s="2" t="inlineStr"/>
+      <c r="AG145" s="2" t="inlineStr"/>
+      <c r="AH145" s="2" t="inlineStr"/>
+      <c r="AI145" s="2" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -18833,6 +19583,11 @@
       <c r="AB146" s="2" t="inlineStr"/>
       <c r="AC146" s="2" t="inlineStr"/>
       <c r="AD146" s="2" t="inlineStr"/>
+      <c r="AE146" s="2" t="inlineStr"/>
+      <c r="AF146" s="2" t="inlineStr"/>
+      <c r="AG146" s="2" t="inlineStr"/>
+      <c r="AH146" s="2" t="inlineStr"/>
+      <c r="AI146" s="2" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -18959,6 +19714,11 @@
       <c r="AB147" s="2" t="inlineStr"/>
       <c r="AC147" s="2" t="inlineStr"/>
       <c r="AD147" s="2" t="inlineStr"/>
+      <c r="AE147" s="2" t="inlineStr"/>
+      <c r="AF147" s="2" t="inlineStr"/>
+      <c r="AG147" s="2" t="inlineStr"/>
+      <c r="AH147" s="2" t="inlineStr"/>
+      <c r="AI147" s="2" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -19085,6 +19845,11 @@
       <c r="AB148" s="2" t="inlineStr"/>
       <c r="AC148" s="2" t="inlineStr"/>
       <c r="AD148" s="2" t="inlineStr"/>
+      <c r="AE148" s="2" t="inlineStr"/>
+      <c r="AF148" s="2" t="inlineStr"/>
+      <c r="AG148" s="2" t="inlineStr"/>
+      <c r="AH148" s="2" t="inlineStr"/>
+      <c r="AI148" s="2" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -19211,6 +19976,11 @@
       <c r="AB149" s="2" t="inlineStr"/>
       <c r="AC149" s="2" t="inlineStr"/>
       <c r="AD149" s="2" t="inlineStr"/>
+      <c r="AE149" s="2" t="inlineStr"/>
+      <c r="AF149" s="2" t="inlineStr"/>
+      <c r="AG149" s="2" t="inlineStr"/>
+      <c r="AH149" s="2" t="inlineStr"/>
+      <c r="AI149" s="2" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -19337,6 +20107,11 @@
       <c r="AB150" s="2" t="inlineStr"/>
       <c r="AC150" s="2" t="inlineStr"/>
       <c r="AD150" s="2" t="inlineStr"/>
+      <c r="AE150" s="2" t="inlineStr"/>
+      <c r="AF150" s="2" t="inlineStr"/>
+      <c r="AG150" s="2" t="inlineStr"/>
+      <c r="AH150" s="2" t="inlineStr"/>
+      <c r="AI150" s="2" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -19463,6 +20238,11 @@
       <c r="AB151" s="2" t="inlineStr"/>
       <c r="AC151" s="2" t="inlineStr"/>
       <c r="AD151" s="2" t="inlineStr"/>
+      <c r="AE151" s="2" t="inlineStr"/>
+      <c r="AF151" s="2" t="inlineStr"/>
+      <c r="AG151" s="2" t="inlineStr"/>
+      <c r="AH151" s="2" t="inlineStr"/>
+      <c r="AI151" s="2" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -19589,6 +20369,11 @@
       <c r="AB152" s="2" t="inlineStr"/>
       <c r="AC152" s="2" t="inlineStr"/>
       <c r="AD152" s="2" t="inlineStr"/>
+      <c r="AE152" s="2" t="inlineStr"/>
+      <c r="AF152" s="2" t="inlineStr"/>
+      <c r="AG152" s="2" t="inlineStr"/>
+      <c r="AH152" s="2" t="inlineStr"/>
+      <c r="AI152" s="2" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -19715,6 +20500,11 @@
       <c r="AB153" s="2" t="inlineStr"/>
       <c r="AC153" s="2" t="inlineStr"/>
       <c r="AD153" s="2" t="inlineStr"/>
+      <c r="AE153" s="2" t="inlineStr"/>
+      <c r="AF153" s="2" t="inlineStr"/>
+      <c r="AG153" s="2" t="inlineStr"/>
+      <c r="AH153" s="2" t="inlineStr"/>
+      <c r="AI153" s="2" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -19841,6 +20631,11 @@
       <c r="AB154" s="2" t="inlineStr"/>
       <c r="AC154" s="2" t="inlineStr"/>
       <c r="AD154" s="2" t="inlineStr"/>
+      <c r="AE154" s="2" t="inlineStr"/>
+      <c r="AF154" s="2" t="inlineStr"/>
+      <c r="AG154" s="2" t="inlineStr"/>
+      <c r="AH154" s="2" t="inlineStr"/>
+      <c r="AI154" s="2" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -19967,6 +20762,11 @@
       <c r="AB155" s="2" t="inlineStr"/>
       <c r="AC155" s="2" t="inlineStr"/>
       <c r="AD155" s="2" t="inlineStr"/>
+      <c r="AE155" s="2" t="inlineStr"/>
+      <c r="AF155" s="2" t="inlineStr"/>
+      <c r="AG155" s="2" t="inlineStr"/>
+      <c r="AH155" s="2" t="inlineStr"/>
+      <c r="AI155" s="2" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -20093,6 +20893,11 @@
       <c r="AB156" s="2" t="inlineStr"/>
       <c r="AC156" s="2" t="inlineStr"/>
       <c r="AD156" s="2" t="inlineStr"/>
+      <c r="AE156" s="2" t="inlineStr"/>
+      <c r="AF156" s="2" t="inlineStr"/>
+      <c r="AG156" s="2" t="inlineStr"/>
+      <c r="AH156" s="2" t="inlineStr"/>
+      <c r="AI156" s="2" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -20219,6 +21024,11 @@
       <c r="AB157" s="2" t="inlineStr"/>
       <c r="AC157" s="2" t="inlineStr"/>
       <c r="AD157" s="2" t="inlineStr"/>
+      <c r="AE157" s="2" t="inlineStr"/>
+      <c r="AF157" s="2" t="inlineStr"/>
+      <c r="AG157" s="2" t="inlineStr"/>
+      <c r="AH157" s="2" t="inlineStr"/>
+      <c r="AI157" s="2" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -20345,6 +21155,11 @@
       <c r="AB158" s="2" t="inlineStr"/>
       <c r="AC158" s="2" t="inlineStr"/>
       <c r="AD158" s="2" t="inlineStr"/>
+      <c r="AE158" s="2" t="inlineStr"/>
+      <c r="AF158" s="2" t="inlineStr"/>
+      <c r="AG158" s="2" t="inlineStr"/>
+      <c r="AH158" s="2" t="inlineStr"/>
+      <c r="AI158" s="2" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -20471,6 +21286,11 @@
       <c r="AB159" s="2" t="inlineStr"/>
       <c r="AC159" s="2" t="inlineStr"/>
       <c r="AD159" s="2" t="inlineStr"/>
+      <c r="AE159" s="2" t="inlineStr"/>
+      <c r="AF159" s="2" t="inlineStr"/>
+      <c r="AG159" s="2" t="inlineStr"/>
+      <c r="AH159" s="2" t="inlineStr"/>
+      <c r="AI159" s="2" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -20597,6 +21417,11 @@
       <c r="AB160" s="2" t="inlineStr"/>
       <c r="AC160" s="2" t="inlineStr"/>
       <c r="AD160" s="2" t="inlineStr"/>
+      <c r="AE160" s="2" t="inlineStr"/>
+      <c r="AF160" s="2" t="inlineStr"/>
+      <c r="AG160" s="2" t="inlineStr"/>
+      <c r="AH160" s="2" t="inlineStr"/>
+      <c r="AI160" s="2" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -20723,6 +21548,11 @@
       <c r="AB161" s="2" t="inlineStr"/>
       <c r="AC161" s="2" t="inlineStr"/>
       <c r="AD161" s="2" t="inlineStr"/>
+      <c r="AE161" s="2" t="inlineStr"/>
+      <c r="AF161" s="2" t="inlineStr"/>
+      <c r="AG161" s="2" t="inlineStr"/>
+      <c r="AH161" s="2" t="inlineStr"/>
+      <c r="AI161" s="2" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -20849,6 +21679,11 @@
       <c r="AB162" s="2" t="inlineStr"/>
       <c r="AC162" s="2" t="inlineStr"/>
       <c r="AD162" s="2" t="inlineStr"/>
+      <c r="AE162" s="2" t="inlineStr"/>
+      <c r="AF162" s="2" t="inlineStr"/>
+      <c r="AG162" s="2" t="inlineStr"/>
+      <c r="AH162" s="2" t="inlineStr"/>
+      <c r="AI162" s="2" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -20975,6 +21810,11 @@
       <c r="AB163" s="2" t="inlineStr"/>
       <c r="AC163" s="2" t="inlineStr"/>
       <c r="AD163" s="2" t="inlineStr"/>
+      <c r="AE163" s="2" t="inlineStr"/>
+      <c r="AF163" s="2" t="inlineStr"/>
+      <c r="AG163" s="2" t="inlineStr"/>
+      <c r="AH163" s="2" t="inlineStr"/>
+      <c r="AI163" s="2" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -21101,6 +21941,11 @@
       <c r="AB164" s="2" t="inlineStr"/>
       <c r="AC164" s="2" t="inlineStr"/>
       <c r="AD164" s="2" t="inlineStr"/>
+      <c r="AE164" s="2" t="inlineStr"/>
+      <c r="AF164" s="2" t="inlineStr"/>
+      <c r="AG164" s="2" t="inlineStr"/>
+      <c r="AH164" s="2" t="inlineStr"/>
+      <c r="AI164" s="2" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -21227,6 +22072,11 @@
       <c r="AB165" s="2" t="inlineStr"/>
       <c r="AC165" s="2" t="inlineStr"/>
       <c r="AD165" s="2" t="inlineStr"/>
+      <c r="AE165" s="2" t="inlineStr"/>
+      <c r="AF165" s="2" t="inlineStr"/>
+      <c r="AG165" s="2" t="inlineStr"/>
+      <c r="AH165" s="2" t="inlineStr"/>
+      <c r="AI165" s="2" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -21353,6 +22203,11 @@
       <c r="AB166" s="2" t="inlineStr"/>
       <c r="AC166" s="2" t="inlineStr"/>
       <c r="AD166" s="2" t="inlineStr"/>
+      <c r="AE166" s="2" t="inlineStr"/>
+      <c r="AF166" s="2" t="inlineStr"/>
+      <c r="AG166" s="2" t="inlineStr"/>
+      <c r="AH166" s="2" t="inlineStr"/>
+      <c r="AI166" s="2" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -21479,6 +22334,11 @@
       <c r="AB167" s="2" t="inlineStr"/>
       <c r="AC167" s="2" t="inlineStr"/>
       <c r="AD167" s="2" t="inlineStr"/>
+      <c r="AE167" s="2" t="inlineStr"/>
+      <c r="AF167" s="2" t="inlineStr"/>
+      <c r="AG167" s="2" t="inlineStr"/>
+      <c r="AH167" s="2" t="inlineStr"/>
+      <c r="AI167" s="2" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -21605,6 +22465,11 @@
       <c r="AB168" s="2" t="inlineStr"/>
       <c r="AC168" s="2" t="inlineStr"/>
       <c r="AD168" s="2" t="inlineStr"/>
+      <c r="AE168" s="2" t="inlineStr"/>
+      <c r="AF168" s="2" t="inlineStr"/>
+      <c r="AG168" s="2" t="inlineStr"/>
+      <c r="AH168" s="2" t="inlineStr"/>
+      <c r="AI168" s="2" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -21731,6 +22596,11 @@
       <c r="AB169" s="2" t="inlineStr"/>
       <c r="AC169" s="2" t="inlineStr"/>
       <c r="AD169" s="2" t="inlineStr"/>
+      <c r="AE169" s="2" t="inlineStr"/>
+      <c r="AF169" s="2" t="inlineStr"/>
+      <c r="AG169" s="2" t="inlineStr"/>
+      <c r="AH169" s="2" t="inlineStr"/>
+      <c r="AI169" s="2" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -21857,6 +22727,11 @@
       <c r="AB170" s="2" t="inlineStr"/>
       <c r="AC170" s="2" t="inlineStr"/>
       <c r="AD170" s="2" t="inlineStr"/>
+      <c r="AE170" s="2" t="inlineStr"/>
+      <c r="AF170" s="2" t="inlineStr"/>
+      <c r="AG170" s="2" t="inlineStr"/>
+      <c r="AH170" s="2" t="inlineStr"/>
+      <c r="AI170" s="2" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -21983,6 +22858,11 @@
       <c r="AB171" s="2" t="inlineStr"/>
       <c r="AC171" s="2" t="inlineStr"/>
       <c r="AD171" s="2" t="inlineStr"/>
+      <c r="AE171" s="2" t="inlineStr"/>
+      <c r="AF171" s="2" t="inlineStr"/>
+      <c r="AG171" s="2" t="inlineStr"/>
+      <c r="AH171" s="2" t="inlineStr"/>
+      <c r="AI171" s="2" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -22109,6 +22989,11 @@
       <c r="AB172" s="2" t="inlineStr"/>
       <c r="AC172" s="2" t="inlineStr"/>
       <c r="AD172" s="2" t="inlineStr"/>
+      <c r="AE172" s="2" t="inlineStr"/>
+      <c r="AF172" s="2" t="inlineStr"/>
+      <c r="AG172" s="2" t="inlineStr"/>
+      <c r="AH172" s="2" t="inlineStr"/>
+      <c r="AI172" s="2" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -22235,6 +23120,11 @@
       <c r="AB173" s="2" t="inlineStr"/>
       <c r="AC173" s="2" t="inlineStr"/>
       <c r="AD173" s="2" t="inlineStr"/>
+      <c r="AE173" s="2" t="inlineStr"/>
+      <c r="AF173" s="2" t="inlineStr"/>
+      <c r="AG173" s="2" t="inlineStr"/>
+      <c r="AH173" s="2" t="inlineStr"/>
+      <c r="AI173" s="2" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -22361,6 +23251,11 @@
       <c r="AB174" s="2" t="inlineStr"/>
       <c r="AC174" s="2" t="inlineStr"/>
       <c r="AD174" s="2" t="inlineStr"/>
+      <c r="AE174" s="2" t="inlineStr"/>
+      <c r="AF174" s="2" t="inlineStr"/>
+      <c r="AG174" s="2" t="inlineStr"/>
+      <c r="AH174" s="2" t="inlineStr"/>
+      <c r="AI174" s="2" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -22487,6 +23382,11 @@
       <c r="AB175" s="2" t="inlineStr"/>
       <c r="AC175" s="2" t="inlineStr"/>
       <c r="AD175" s="2" t="inlineStr"/>
+      <c r="AE175" s="2" t="inlineStr"/>
+      <c r="AF175" s="2" t="inlineStr"/>
+      <c r="AG175" s="2" t="inlineStr"/>
+      <c r="AH175" s="2" t="inlineStr"/>
+      <c r="AI175" s="2" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -22613,6 +23513,11 @@
       <c r="AB176" s="2" t="inlineStr"/>
       <c r="AC176" s="2" t="inlineStr"/>
       <c r="AD176" s="2" t="inlineStr"/>
+      <c r="AE176" s="2" t="inlineStr"/>
+      <c r="AF176" s="2" t="inlineStr"/>
+      <c r="AG176" s="2" t="inlineStr"/>
+      <c r="AH176" s="2" t="inlineStr"/>
+      <c r="AI176" s="2" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
@@ -22739,6 +23644,11 @@
       <c r="AB177" s="2" t="inlineStr"/>
       <c r="AC177" s="2" t="inlineStr"/>
       <c r="AD177" s="2" t="inlineStr"/>
+      <c r="AE177" s="2" t="inlineStr"/>
+      <c r="AF177" s="2" t="inlineStr"/>
+      <c r="AG177" s="2" t="inlineStr"/>
+      <c r="AH177" s="2" t="inlineStr"/>
+      <c r="AI177" s="2" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -22865,6 +23775,11 @@
       <c r="AB178" s="2" t="inlineStr"/>
       <c r="AC178" s="2" t="inlineStr"/>
       <c r="AD178" s="2" t="inlineStr"/>
+      <c r="AE178" s="2" t="inlineStr"/>
+      <c r="AF178" s="2" t="inlineStr"/>
+      <c r="AG178" s="2" t="inlineStr"/>
+      <c r="AH178" s="2" t="inlineStr"/>
+      <c r="AI178" s="2" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -22991,6 +23906,11 @@
       <c r="AB179" s="2" t="inlineStr"/>
       <c r="AC179" s="2" t="inlineStr"/>
       <c r="AD179" s="2" t="inlineStr"/>
+      <c r="AE179" s="2" t="inlineStr"/>
+      <c r="AF179" s="2" t="inlineStr"/>
+      <c r="AG179" s="2" t="inlineStr"/>
+      <c r="AH179" s="2" t="inlineStr"/>
+      <c r="AI179" s="2" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -23117,6 +24037,11 @@
       <c r="AB180" s="2" t="inlineStr"/>
       <c r="AC180" s="2" t="inlineStr"/>
       <c r="AD180" s="2" t="inlineStr"/>
+      <c r="AE180" s="2" t="inlineStr"/>
+      <c r="AF180" s="2" t="inlineStr"/>
+      <c r="AG180" s="2" t="inlineStr"/>
+      <c r="AH180" s="2" t="inlineStr"/>
+      <c r="AI180" s="2" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -23243,6 +24168,11 @@
       <c r="AB181" s="2" t="inlineStr"/>
       <c r="AC181" s="2" t="inlineStr"/>
       <c r="AD181" s="2" t="inlineStr"/>
+      <c r="AE181" s="2" t="inlineStr"/>
+      <c r="AF181" s="2" t="inlineStr"/>
+      <c r="AG181" s="2" t="inlineStr"/>
+      <c r="AH181" s="2" t="inlineStr"/>
+      <c r="AI181" s="2" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -23369,6 +24299,11 @@
       <c r="AB182" s="2" t="inlineStr"/>
       <c r="AC182" s="2" t="inlineStr"/>
       <c r="AD182" s="2" t="inlineStr"/>
+      <c r="AE182" s="2" t="inlineStr"/>
+      <c r="AF182" s="2" t="inlineStr"/>
+      <c r="AG182" s="2" t="inlineStr"/>
+      <c r="AH182" s="2" t="inlineStr"/>
+      <c r="AI182" s="2" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
@@ -23495,6 +24430,11 @@
       <c r="AB183" s="2" t="inlineStr"/>
       <c r="AC183" s="2" t="inlineStr"/>
       <c r="AD183" s="2" t="inlineStr"/>
+      <c r="AE183" s="2" t="inlineStr"/>
+      <c r="AF183" s="2" t="inlineStr"/>
+      <c r="AG183" s="2" t="inlineStr"/>
+      <c r="AH183" s="2" t="inlineStr"/>
+      <c r="AI183" s="2" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -23621,6 +24561,11 @@
       <c r="AB184" s="2" t="inlineStr"/>
       <c r="AC184" s="2" t="inlineStr"/>
       <c r="AD184" s="2" t="inlineStr"/>
+      <c r="AE184" s="2" t="inlineStr"/>
+      <c r="AF184" s="2" t="inlineStr"/>
+      <c r="AG184" s="2" t="inlineStr"/>
+      <c r="AH184" s="2" t="inlineStr"/>
+      <c r="AI184" s="2" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
@@ -23747,6 +24692,11 @@
       <c r="AB185" s="2" t="inlineStr"/>
       <c r="AC185" s="2" t="inlineStr"/>
       <c r="AD185" s="2" t="inlineStr"/>
+      <c r="AE185" s="2" t="inlineStr"/>
+      <c r="AF185" s="2" t="inlineStr"/>
+      <c r="AG185" s="2" t="inlineStr"/>
+      <c r="AH185" s="2" t="inlineStr"/>
+      <c r="AI185" s="2" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -23873,6 +24823,11 @@
       <c r="AB186" s="2" t="inlineStr"/>
       <c r="AC186" s="2" t="inlineStr"/>
       <c r="AD186" s="2" t="inlineStr"/>
+      <c r="AE186" s="2" t="inlineStr"/>
+      <c r="AF186" s="2" t="inlineStr"/>
+      <c r="AG186" s="2" t="inlineStr"/>
+      <c r="AH186" s="2" t="inlineStr"/>
+      <c r="AI186" s="2" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
@@ -23999,6 +24954,11 @@
       <c r="AB187" s="2" t="inlineStr"/>
       <c r="AC187" s="2" t="inlineStr"/>
       <c r="AD187" s="2" t="inlineStr"/>
+      <c r="AE187" s="2" t="inlineStr"/>
+      <c r="AF187" s="2" t="inlineStr"/>
+      <c r="AG187" s="2" t="inlineStr"/>
+      <c r="AH187" s="2" t="inlineStr"/>
+      <c r="AI187" s="2" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -24125,6 +25085,11 @@
       <c r="AB188" s="2" t="inlineStr"/>
       <c r="AC188" s="2" t="inlineStr"/>
       <c r="AD188" s="2" t="inlineStr"/>
+      <c r="AE188" s="2" t="inlineStr"/>
+      <c r="AF188" s="2" t="inlineStr"/>
+      <c r="AG188" s="2" t="inlineStr"/>
+      <c r="AH188" s="2" t="inlineStr"/>
+      <c r="AI188" s="2" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
@@ -24251,6 +25216,11 @@
       <c r="AB189" s="2" t="inlineStr"/>
       <c r="AC189" s="2" t="inlineStr"/>
       <c r="AD189" s="2" t="inlineStr"/>
+      <c r="AE189" s="2" t="inlineStr"/>
+      <c r="AF189" s="2" t="inlineStr"/>
+      <c r="AG189" s="2" t="inlineStr"/>
+      <c r="AH189" s="2" t="inlineStr"/>
+      <c r="AI189" s="2" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -24377,6 +25347,11 @@
       <c r="AB190" s="2" t="inlineStr"/>
       <c r="AC190" s="2" t="inlineStr"/>
       <c r="AD190" s="2" t="inlineStr"/>
+      <c r="AE190" s="2" t="inlineStr"/>
+      <c r="AF190" s="2" t="inlineStr"/>
+      <c r="AG190" s="2" t="inlineStr"/>
+      <c r="AH190" s="2" t="inlineStr"/>
+      <c r="AI190" s="2" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
@@ -24503,6 +25478,11 @@
       <c r="AB191" s="2" t="inlineStr"/>
       <c r="AC191" s="2" t="inlineStr"/>
       <c r="AD191" s="2" t="inlineStr"/>
+      <c r="AE191" s="2" t="inlineStr"/>
+      <c r="AF191" s="2" t="inlineStr"/>
+      <c r="AG191" s="2" t="inlineStr"/>
+      <c r="AH191" s="2" t="inlineStr"/>
+      <c r="AI191" s="2" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -24629,6 +25609,11 @@
       <c r="AB192" s="2" t="inlineStr"/>
       <c r="AC192" s="2" t="inlineStr"/>
       <c r="AD192" s="2" t="inlineStr"/>
+      <c r="AE192" s="2" t="inlineStr"/>
+      <c r="AF192" s="2" t="inlineStr"/>
+      <c r="AG192" s="2" t="inlineStr"/>
+      <c r="AH192" s="2" t="inlineStr"/>
+      <c r="AI192" s="2" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
@@ -24755,6 +25740,11 @@
       <c r="AB193" s="2" t="inlineStr"/>
       <c r="AC193" s="2" t="inlineStr"/>
       <c r="AD193" s="2" t="inlineStr"/>
+      <c r="AE193" s="2" t="inlineStr"/>
+      <c r="AF193" s="2" t="inlineStr"/>
+      <c r="AG193" s="2" t="inlineStr"/>
+      <c r="AH193" s="2" t="inlineStr"/>
+      <c r="AI193" s="2" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -24881,6 +25871,11 @@
       <c r="AB194" s="2" t="inlineStr"/>
       <c r="AC194" s="2" t="inlineStr"/>
       <c r="AD194" s="2" t="inlineStr"/>
+      <c r="AE194" s="2" t="inlineStr"/>
+      <c r="AF194" s="2" t="inlineStr"/>
+      <c r="AG194" s="2" t="inlineStr"/>
+      <c r="AH194" s="2" t="inlineStr"/>
+      <c r="AI194" s="2" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
@@ -25007,6 +26002,11 @@
       <c r="AB195" s="2" t="inlineStr"/>
       <c r="AC195" s="2" t="inlineStr"/>
       <c r="AD195" s="2" t="inlineStr"/>
+      <c r="AE195" s="2" t="inlineStr"/>
+      <c r="AF195" s="2" t="inlineStr"/>
+      <c r="AG195" s="2" t="inlineStr"/>
+      <c r="AH195" s="2" t="inlineStr"/>
+      <c r="AI195" s="2" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
@@ -25133,6 +26133,11 @@
       <c r="AB196" s="2" t="inlineStr"/>
       <c r="AC196" s="2" t="inlineStr"/>
       <c r="AD196" s="2" t="inlineStr"/>
+      <c r="AE196" s="2" t="inlineStr"/>
+      <c r="AF196" s="2" t="inlineStr"/>
+      <c r="AG196" s="2" t="inlineStr"/>
+      <c r="AH196" s="2" t="inlineStr"/>
+      <c r="AI196" s="2" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
@@ -25259,6 +26264,11 @@
       <c r="AB197" s="2" t="inlineStr"/>
       <c r="AC197" s="2" t="inlineStr"/>
       <c r="AD197" s="2" t="inlineStr"/>
+      <c r="AE197" s="2" t="inlineStr"/>
+      <c r="AF197" s="2" t="inlineStr"/>
+      <c r="AG197" s="2" t="inlineStr"/>
+      <c r="AH197" s="2" t="inlineStr"/>
+      <c r="AI197" s="2" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -25385,6 +26395,11 @@
       <c r="AB198" s="2" t="inlineStr"/>
       <c r="AC198" s="2" t="inlineStr"/>
       <c r="AD198" s="2" t="inlineStr"/>
+      <c r="AE198" s="2" t="inlineStr"/>
+      <c r="AF198" s="2" t="inlineStr"/>
+      <c r="AG198" s="2" t="inlineStr"/>
+      <c r="AH198" s="2" t="inlineStr"/>
+      <c r="AI198" s="2" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
@@ -25511,6 +26526,11 @@
       <c r="AB199" s="2" t="inlineStr"/>
       <c r="AC199" s="2" t="inlineStr"/>
       <c r="AD199" s="2" t="inlineStr"/>
+      <c r="AE199" s="2" t="inlineStr"/>
+      <c r="AF199" s="2" t="inlineStr"/>
+      <c r="AG199" s="2" t="inlineStr"/>
+      <c r="AH199" s="2" t="inlineStr"/>
+      <c r="AI199" s="2" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -25637,6 +26657,11 @@
       <c r="AB200" s="2" t="inlineStr"/>
       <c r="AC200" s="2" t="inlineStr"/>
       <c r="AD200" s="2" t="inlineStr"/>
+      <c r="AE200" s="2" t="inlineStr"/>
+      <c r="AF200" s="2" t="inlineStr"/>
+      <c r="AG200" s="2" t="inlineStr"/>
+      <c r="AH200" s="2" t="inlineStr"/>
+      <c r="AI200" s="2" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" s="4" t="inlineStr">
@@ -25769,6 +26794,11 @@
           <t>API call failed (api_payload_dump) → retried → APPROVED</t>
         </is>
       </c>
+      <c r="AE201" s="4" t="inlineStr"/>
+      <c r="AF201" s="4" t="inlineStr"/>
+      <c r="AG201" s="4" t="inlineStr"/>
+      <c r="AH201" s="4" t="inlineStr"/>
+      <c r="AI201" s="4" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -25895,6 +26925,11 @@
       <c r="AB202" s="2" t="inlineStr"/>
       <c r="AC202" s="2" t="inlineStr"/>
       <c r="AD202" s="2" t="inlineStr"/>
+      <c r="AE202" s="2" t="inlineStr"/>
+      <c r="AF202" s="2" t="inlineStr"/>
+      <c r="AG202" s="2" t="inlineStr"/>
+      <c r="AH202" s="2" t="inlineStr"/>
+      <c r="AI202" s="2" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
@@ -26021,6 +27056,11 @@
       <c r="AB203" s="2" t="inlineStr"/>
       <c r="AC203" s="2" t="inlineStr"/>
       <c r="AD203" s="2" t="inlineStr"/>
+      <c r="AE203" s="2" t="inlineStr"/>
+      <c r="AF203" s="2" t="inlineStr"/>
+      <c r="AG203" s="2" t="inlineStr"/>
+      <c r="AH203" s="2" t="inlineStr"/>
+      <c r="AI203" s="2" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -26147,6 +27187,11 @@
       <c r="AB204" s="2" t="inlineStr"/>
       <c r="AC204" s="2" t="inlineStr"/>
       <c r="AD204" s="2" t="inlineStr"/>
+      <c r="AE204" s="2" t="inlineStr"/>
+      <c r="AF204" s="2" t="inlineStr"/>
+      <c r="AG204" s="2" t="inlineStr"/>
+      <c r="AH204" s="2" t="inlineStr"/>
+      <c r="AI204" s="2" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" s="4" t="inlineStr">
@@ -26279,6 +27324,11 @@
           <t>API call failed (api_payload_dump) → retried → APPROVED</t>
         </is>
       </c>
+      <c r="AE205" s="4" t="inlineStr"/>
+      <c r="AF205" s="4" t="inlineStr"/>
+      <c r="AG205" s="4" t="inlineStr"/>
+      <c r="AH205" s="4" t="inlineStr"/>
+      <c r="AI205" s="4" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -26405,6 +27455,11 @@
       <c r="AB206" s="2" t="inlineStr"/>
       <c r="AC206" s="2" t="inlineStr"/>
       <c r="AD206" s="2" t="inlineStr"/>
+      <c r="AE206" s="2" t="inlineStr"/>
+      <c r="AF206" s="2" t="inlineStr"/>
+      <c r="AG206" s="2" t="inlineStr"/>
+      <c r="AH206" s="2" t="inlineStr"/>
+      <c r="AI206" s="2" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
@@ -26531,6 +27586,11 @@
       <c r="AB207" s="2" t="inlineStr"/>
       <c r="AC207" s="2" t="inlineStr"/>
       <c r="AD207" s="2" t="inlineStr"/>
+      <c r="AE207" s="2" t="inlineStr"/>
+      <c r="AF207" s="2" t="inlineStr"/>
+      <c r="AG207" s="2" t="inlineStr"/>
+      <c r="AH207" s="2" t="inlineStr"/>
+      <c r="AI207" s="2" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
@@ -26657,6 +27717,11 @@
       <c r="AB208" s="2" t="inlineStr"/>
       <c r="AC208" s="2" t="inlineStr"/>
       <c r="AD208" s="2" t="inlineStr"/>
+      <c r="AE208" s="2" t="inlineStr"/>
+      <c r="AF208" s="2" t="inlineStr"/>
+      <c r="AG208" s="2" t="inlineStr"/>
+      <c r="AH208" s="2" t="inlineStr"/>
+      <c r="AI208" s="2" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
@@ -26783,6 +27848,11 @@
       <c r="AB209" s="2" t="inlineStr"/>
       <c r="AC209" s="2" t="inlineStr"/>
       <c r="AD209" s="2" t="inlineStr"/>
+      <c r="AE209" s="2" t="inlineStr"/>
+      <c r="AF209" s="2" t="inlineStr"/>
+      <c r="AG209" s="2" t="inlineStr"/>
+      <c r="AH209" s="2" t="inlineStr"/>
+      <c r="AI209" s="2" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -26909,6 +27979,11 @@
       <c r="AB210" s="2" t="inlineStr"/>
       <c r="AC210" s="2" t="inlineStr"/>
       <c r="AD210" s="2" t="inlineStr"/>
+      <c r="AE210" s="2" t="inlineStr"/>
+      <c r="AF210" s="2" t="inlineStr"/>
+      <c r="AG210" s="2" t="inlineStr"/>
+      <c r="AH210" s="2" t="inlineStr"/>
+      <c r="AI210" s="2" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
@@ -27035,6 +28110,11 @@
       <c r="AB211" s="2" t="inlineStr"/>
       <c r="AC211" s="2" t="inlineStr"/>
       <c r="AD211" s="2" t="inlineStr"/>
+      <c r="AE211" s="2" t="inlineStr"/>
+      <c r="AF211" s="2" t="inlineStr"/>
+      <c r="AG211" s="2" t="inlineStr"/>
+      <c r="AH211" s="2" t="inlineStr"/>
+      <c r="AI211" s="2" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
@@ -27161,6 +28241,11 @@
       <c r="AB212" s="2" t="inlineStr"/>
       <c r="AC212" s="2" t="inlineStr"/>
       <c r="AD212" s="2" t="inlineStr"/>
+      <c r="AE212" s="2" t="inlineStr"/>
+      <c r="AF212" s="2" t="inlineStr"/>
+      <c r="AG212" s="2" t="inlineStr"/>
+      <c r="AH212" s="2" t="inlineStr"/>
+      <c r="AI212" s="2" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
@@ -27287,6 +28372,11 @@
       <c r="AB213" s="2" t="inlineStr"/>
       <c r="AC213" s="2" t="inlineStr"/>
       <c r="AD213" s="2" t="inlineStr"/>
+      <c r="AE213" s="2" t="inlineStr"/>
+      <c r="AF213" s="2" t="inlineStr"/>
+      <c r="AG213" s="2" t="inlineStr"/>
+      <c r="AH213" s="2" t="inlineStr"/>
+      <c r="AI213" s="2" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
@@ -27413,6 +28503,11 @@
       <c r="AB214" s="2" t="inlineStr"/>
       <c r="AC214" s="2" t="inlineStr"/>
       <c r="AD214" s="2" t="inlineStr"/>
+      <c r="AE214" s="2" t="inlineStr"/>
+      <c r="AF214" s="2" t="inlineStr"/>
+      <c r="AG214" s="2" t="inlineStr"/>
+      <c r="AH214" s="2" t="inlineStr"/>
+      <c r="AI214" s="2" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
@@ -27539,6 +28634,11 @@
       <c r="AB215" s="2" t="inlineStr"/>
       <c r="AC215" s="2" t="inlineStr"/>
       <c r="AD215" s="2" t="inlineStr"/>
+      <c r="AE215" s="2" t="inlineStr"/>
+      <c r="AF215" s="2" t="inlineStr"/>
+      <c r="AG215" s="2" t="inlineStr"/>
+      <c r="AH215" s="2" t="inlineStr"/>
+      <c r="AI215" s="2" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
@@ -27665,6 +28765,11 @@
       <c r="AB216" s="2" t="inlineStr"/>
       <c r="AC216" s="2" t="inlineStr"/>
       <c r="AD216" s="2" t="inlineStr"/>
+      <c r="AE216" s="2" t="inlineStr"/>
+      <c r="AF216" s="2" t="inlineStr"/>
+      <c r="AG216" s="2" t="inlineStr"/>
+      <c r="AH216" s="2" t="inlineStr"/>
+      <c r="AI216" s="2" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
@@ -27791,6 +28896,11 @@
       <c r="AB217" s="2" t="inlineStr"/>
       <c r="AC217" s="2" t="inlineStr"/>
       <c r="AD217" s="2" t="inlineStr"/>
+      <c r="AE217" s="2" t="inlineStr"/>
+      <c r="AF217" s="2" t="inlineStr"/>
+      <c r="AG217" s="2" t="inlineStr"/>
+      <c r="AH217" s="2" t="inlineStr"/>
+      <c r="AI217" s="2" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
@@ -27917,6 +29027,11 @@
       <c r="AB218" s="2" t="inlineStr"/>
       <c r="AC218" s="2" t="inlineStr"/>
       <c r="AD218" s="2" t="inlineStr"/>
+      <c r="AE218" s="2" t="inlineStr"/>
+      <c r="AF218" s="2" t="inlineStr"/>
+      <c r="AG218" s="2" t="inlineStr"/>
+      <c r="AH218" s="2" t="inlineStr"/>
+      <c r="AI218" s="2" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
@@ -28043,6 +29158,11 @@
       <c r="AB219" s="2" t="inlineStr"/>
       <c r="AC219" s="2" t="inlineStr"/>
       <c r="AD219" s="2" t="inlineStr"/>
+      <c r="AE219" s="2" t="inlineStr"/>
+      <c r="AF219" s="2" t="inlineStr"/>
+      <c r="AG219" s="2" t="inlineStr"/>
+      <c r="AH219" s="2" t="inlineStr"/>
+      <c r="AI219" s="2" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -28169,6 +29289,11 @@
       <c r="AB220" s="2" t="inlineStr"/>
       <c r="AC220" s="2" t="inlineStr"/>
       <c r="AD220" s="2" t="inlineStr"/>
+      <c r="AE220" s="2" t="inlineStr"/>
+      <c r="AF220" s="2" t="inlineStr"/>
+      <c r="AG220" s="2" t="inlineStr"/>
+      <c r="AH220" s="2" t="inlineStr"/>
+      <c r="AI220" s="2" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
@@ -28295,6 +29420,11 @@
       <c r="AB221" s="2" t="inlineStr"/>
       <c r="AC221" s="2" t="inlineStr"/>
       <c r="AD221" s="2" t="inlineStr"/>
+      <c r="AE221" s="2" t="inlineStr"/>
+      <c r="AF221" s="2" t="inlineStr"/>
+      <c r="AG221" s="2" t="inlineStr"/>
+      <c r="AH221" s="2" t="inlineStr"/>
+      <c r="AI221" s="2" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
@@ -28421,6 +29551,11 @@
       <c r="AB222" s="2" t="inlineStr"/>
       <c r="AC222" s="2" t="inlineStr"/>
       <c r="AD222" s="2" t="inlineStr"/>
+      <c r="AE222" s="2" t="inlineStr"/>
+      <c r="AF222" s="2" t="inlineStr"/>
+      <c r="AG222" s="2" t="inlineStr"/>
+      <c r="AH222" s="2" t="inlineStr"/>
+      <c r="AI222" s="2" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
@@ -28547,6 +29682,11 @@
       <c r="AB223" s="2" t="inlineStr"/>
       <c r="AC223" s="2" t="inlineStr"/>
       <c r="AD223" s="2" t="inlineStr"/>
+      <c r="AE223" s="2" t="inlineStr"/>
+      <c r="AF223" s="2" t="inlineStr"/>
+      <c r="AG223" s="2" t="inlineStr"/>
+      <c r="AH223" s="2" t="inlineStr"/>
+      <c r="AI223" s="2" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
@@ -28673,6 +29813,11 @@
       <c r="AB224" s="2" t="inlineStr"/>
       <c r="AC224" s="2" t="inlineStr"/>
       <c r="AD224" s="2" t="inlineStr"/>
+      <c r="AE224" s="2" t="inlineStr"/>
+      <c r="AF224" s="2" t="inlineStr"/>
+      <c r="AG224" s="2" t="inlineStr"/>
+      <c r="AH224" s="2" t="inlineStr"/>
+      <c r="AI224" s="2" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
@@ -28799,6 +29944,11 @@
       <c r="AB225" s="2" t="inlineStr"/>
       <c r="AC225" s="2" t="inlineStr"/>
       <c r="AD225" s="2" t="inlineStr"/>
+      <c r="AE225" s="2" t="inlineStr"/>
+      <c r="AF225" s="2" t="inlineStr"/>
+      <c r="AG225" s="2" t="inlineStr"/>
+      <c r="AH225" s="2" t="inlineStr"/>
+      <c r="AI225" s="2" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
@@ -28925,6 +30075,11 @@
       <c r="AB226" s="2" t="inlineStr"/>
       <c r="AC226" s="2" t="inlineStr"/>
       <c r="AD226" s="2" t="inlineStr"/>
+      <c r="AE226" s="2" t="inlineStr"/>
+      <c r="AF226" s="2" t="inlineStr"/>
+      <c r="AG226" s="2" t="inlineStr"/>
+      <c r="AH226" s="2" t="inlineStr"/>
+      <c r="AI226" s="2" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
@@ -29051,6 +30206,11 @@
       <c r="AB227" s="2" t="inlineStr"/>
       <c r="AC227" s="2" t="inlineStr"/>
       <c r="AD227" s="2" t="inlineStr"/>
+      <c r="AE227" s="2" t="inlineStr"/>
+      <c r="AF227" s="2" t="inlineStr"/>
+      <c r="AG227" s="2" t="inlineStr"/>
+      <c r="AH227" s="2" t="inlineStr"/>
+      <c r="AI227" s="2" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
@@ -29177,6 +30337,11 @@
       <c r="AB228" s="2" t="inlineStr"/>
       <c r="AC228" s="2" t="inlineStr"/>
       <c r="AD228" s="2" t="inlineStr"/>
+      <c r="AE228" s="2" t="inlineStr"/>
+      <c r="AF228" s="2" t="inlineStr"/>
+      <c r="AG228" s="2" t="inlineStr"/>
+      <c r="AH228" s="2" t="inlineStr"/>
+      <c r="AI228" s="2" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
@@ -29303,6 +30468,11 @@
       <c r="AB229" s="2" t="inlineStr"/>
       <c r="AC229" s="2" t="inlineStr"/>
       <c r="AD229" s="2" t="inlineStr"/>
+      <c r="AE229" s="2" t="inlineStr"/>
+      <c r="AF229" s="2" t="inlineStr"/>
+      <c r="AG229" s="2" t="inlineStr"/>
+      <c r="AH229" s="2" t="inlineStr"/>
+      <c r="AI229" s="2" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
@@ -29429,6 +30599,11 @@
       <c r="AB230" s="2" t="inlineStr"/>
       <c r="AC230" s="2" t="inlineStr"/>
       <c r="AD230" s="2" t="inlineStr"/>
+      <c r="AE230" s="2" t="inlineStr"/>
+      <c r="AF230" s="2" t="inlineStr"/>
+      <c r="AG230" s="2" t="inlineStr"/>
+      <c r="AH230" s="2" t="inlineStr"/>
+      <c r="AI230" s="2" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
@@ -29555,6 +30730,11 @@
       <c r="AB231" s="2" t="inlineStr"/>
       <c r="AC231" s="2" t="inlineStr"/>
       <c r="AD231" s="2" t="inlineStr"/>
+      <c r="AE231" s="2" t="inlineStr"/>
+      <c r="AF231" s="2" t="inlineStr"/>
+      <c r="AG231" s="2" t="inlineStr"/>
+      <c r="AH231" s="2" t="inlineStr"/>
+      <c r="AI231" s="2" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
@@ -29681,6 +30861,11 @@
       <c r="AB232" s="2" t="inlineStr"/>
       <c r="AC232" s="2" t="inlineStr"/>
       <c r="AD232" s="2" t="inlineStr"/>
+      <c r="AE232" s="2" t="inlineStr"/>
+      <c r="AF232" s="2" t="inlineStr"/>
+      <c r="AG232" s="2" t="inlineStr"/>
+      <c r="AH232" s="2" t="inlineStr"/>
+      <c r="AI232" s="2" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
@@ -29807,6 +30992,11 @@
       <c r="AB233" s="2" t="inlineStr"/>
       <c r="AC233" s="2" t="inlineStr"/>
       <c r="AD233" s="2" t="inlineStr"/>
+      <c r="AE233" s="2" t="inlineStr"/>
+      <c r="AF233" s="2" t="inlineStr"/>
+      <c r="AG233" s="2" t="inlineStr"/>
+      <c r="AH233" s="2" t="inlineStr"/>
+      <c r="AI233" s="2" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
@@ -29933,6 +31123,11 @@
       <c r="AB234" s="2" t="inlineStr"/>
       <c r="AC234" s="2" t="inlineStr"/>
       <c r="AD234" s="2" t="inlineStr"/>
+      <c r="AE234" s="2" t="inlineStr"/>
+      <c r="AF234" s="2" t="inlineStr"/>
+      <c r="AG234" s="2" t="inlineStr"/>
+      <c r="AH234" s="2" t="inlineStr"/>
+      <c r="AI234" s="2" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
@@ -30059,6 +31254,11 @@
       <c r="AB235" s="2" t="inlineStr"/>
       <c r="AC235" s="2" t="inlineStr"/>
       <c r="AD235" s="2" t="inlineStr"/>
+      <c r="AE235" s="2" t="inlineStr"/>
+      <c r="AF235" s="2" t="inlineStr"/>
+      <c r="AG235" s="2" t="inlineStr"/>
+      <c r="AH235" s="2" t="inlineStr"/>
+      <c r="AI235" s="2" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
@@ -30185,6 +31385,11 @@
       <c r="AB236" s="2" t="inlineStr"/>
       <c r="AC236" s="2" t="inlineStr"/>
       <c r="AD236" s="2" t="inlineStr"/>
+      <c r="AE236" s="2" t="inlineStr"/>
+      <c r="AF236" s="2" t="inlineStr"/>
+      <c r="AG236" s="2" t="inlineStr"/>
+      <c r="AH236" s="2" t="inlineStr"/>
+      <c r="AI236" s="2" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
@@ -30311,6 +31516,11 @@
       <c r="AB237" s="2" t="inlineStr"/>
       <c r="AC237" s="2" t="inlineStr"/>
       <c r="AD237" s="2" t="inlineStr"/>
+      <c r="AE237" s="2" t="inlineStr"/>
+      <c r="AF237" s="2" t="inlineStr"/>
+      <c r="AG237" s="2" t="inlineStr"/>
+      <c r="AH237" s="2" t="inlineStr"/>
+      <c r="AI237" s="2" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
@@ -30437,6 +31647,11 @@
       <c r="AB238" s="2" t="inlineStr"/>
       <c r="AC238" s="2" t="inlineStr"/>
       <c r="AD238" s="2" t="inlineStr"/>
+      <c r="AE238" s="2" t="inlineStr"/>
+      <c r="AF238" s="2" t="inlineStr"/>
+      <c r="AG238" s="2" t="inlineStr"/>
+      <c r="AH238" s="2" t="inlineStr"/>
+      <c r="AI238" s="2" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
@@ -30563,6 +31778,11 @@
       <c r="AB239" s="2" t="inlineStr"/>
       <c r="AC239" s="2" t="inlineStr"/>
       <c r="AD239" s="2" t="inlineStr"/>
+      <c r="AE239" s="2" t="inlineStr"/>
+      <c r="AF239" s="2" t="inlineStr"/>
+      <c r="AG239" s="2" t="inlineStr"/>
+      <c r="AH239" s="2" t="inlineStr"/>
+      <c r="AI239" s="2" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
@@ -30689,6 +31909,11 @@
       <c r="AB240" s="2" t="inlineStr"/>
       <c r="AC240" s="2" t="inlineStr"/>
       <c r="AD240" s="2" t="inlineStr"/>
+      <c r="AE240" s="2" t="inlineStr"/>
+      <c r="AF240" s="2" t="inlineStr"/>
+      <c r="AG240" s="2" t="inlineStr"/>
+      <c r="AH240" s="2" t="inlineStr"/>
+      <c r="AI240" s="2" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
@@ -30815,6 +32040,11 @@
       <c r="AB241" s="2" t="inlineStr"/>
       <c r="AC241" s="2" t="inlineStr"/>
       <c r="AD241" s="2" t="inlineStr"/>
+      <c r="AE241" s="2" t="inlineStr"/>
+      <c r="AF241" s="2" t="inlineStr"/>
+      <c r="AG241" s="2" t="inlineStr"/>
+      <c r="AH241" s="2" t="inlineStr"/>
+      <c r="AI241" s="2" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
@@ -30941,6 +32171,11 @@
       <c r="AB242" s="2" t="inlineStr"/>
       <c r="AC242" s="2" t="inlineStr"/>
       <c r="AD242" s="2" t="inlineStr"/>
+      <c r="AE242" s="2" t="inlineStr"/>
+      <c r="AF242" s="2" t="inlineStr"/>
+      <c r="AG242" s="2" t="inlineStr"/>
+      <c r="AH242" s="2" t="inlineStr"/>
+      <c r="AI242" s="2" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
@@ -31067,6 +32302,11 @@
       <c r="AB243" s="2" t="inlineStr"/>
       <c r="AC243" s="2" t="inlineStr"/>
       <c r="AD243" s="2" t="inlineStr"/>
+      <c r="AE243" s="2" t="inlineStr"/>
+      <c r="AF243" s="2" t="inlineStr"/>
+      <c r="AG243" s="2" t="inlineStr"/>
+      <c r="AH243" s="2" t="inlineStr"/>
+      <c r="AI243" s="2" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
@@ -31193,6 +32433,11 @@
       <c r="AB244" s="2" t="inlineStr"/>
       <c r="AC244" s="2" t="inlineStr"/>
       <c r="AD244" s="2" t="inlineStr"/>
+      <c r="AE244" s="2" t="inlineStr"/>
+      <c r="AF244" s="2" t="inlineStr"/>
+      <c r="AG244" s="2" t="inlineStr"/>
+      <c r="AH244" s="2" t="inlineStr"/>
+      <c r="AI244" s="2" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
@@ -31319,9 +32564,14 @@
       <c r="AB245" s="2" t="inlineStr"/>
       <c r="AC245" s="2" t="inlineStr"/>
       <c r="AD245" s="2" t="inlineStr"/>
+      <c r="AE245" s="2" t="inlineStr"/>
+      <c r="AF245" s="2" t="inlineStr"/>
+      <c r="AG245" s="2" t="inlineStr"/>
+      <c r="AH245" s="2" t="inlineStr"/>
+      <c r="AI245" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD245"/>
+  <autoFilter ref="A1:AI245"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -31332,7 +32582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -31345,6 +32595,10 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -31398,6 +32652,26 @@
           <t>Max Duration</t>
         </is>
       </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>API Requests</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>Prompt Tokens</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>Completion Tokens</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>Total Tokens</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -31438,6 +32712,10 @@
           <t>42.5s</t>
         </is>
       </c>
+      <c r="K2" s="6" t="inlineStr"/>
+      <c r="L2" s="6" t="inlineStr"/>
+      <c r="M2" s="6" t="inlineStr"/>
+      <c r="N2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -31478,6 +32756,10 @@
           <t>1m 28.9s</t>
         </is>
       </c>
+      <c r="K3" s="6" t="inlineStr"/>
+      <c r="L3" s="6" t="inlineStr"/>
+      <c r="M3" s="6" t="inlineStr"/>
+      <c r="N3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -31518,6 +32800,10 @@
           <t>25.9s</t>
         </is>
       </c>
+      <c r="K4" s="6" t="inlineStr"/>
+      <c r="L4" s="6" t="inlineStr"/>
+      <c r="M4" s="6" t="inlineStr"/>
+      <c r="N4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -31558,6 +32844,10 @@
           <t>52.5s</t>
         </is>
       </c>
+      <c r="K5" s="6" t="inlineStr"/>
+      <c r="L5" s="6" t="inlineStr"/>
+      <c r="M5" s="6" t="inlineStr"/>
+      <c r="N5" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -31623,7 +32913,7 @@
         <v>24586</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>1498</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="3">
@@ -31691,7 +32981,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr"/>
       <c r="E6" s="6" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7">
@@ -31710,7 +33000,7 @@
         <v>135602</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>132428</v>
+        <v>146730</v>
       </c>
     </row>
     <row r="8">
@@ -31729,7 +33019,7 @@
         <v>21928</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>3641</v>
+        <v>4116</v>
       </c>
     </row>
     <row r="9">
@@ -31748,7 +33038,7 @@
         <v>12256</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>10513</v>
+        <v>11677</v>
       </c>
     </row>
     <row r="10">
@@ -31767,7 +33057,7 @@
         <v>1648</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>1144</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="11">
@@ -31786,7 +33076,7 @@
         <v>1128</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>2018</v>
+        <v>2332</v>
       </c>
     </row>
     <row r="12">

</xml_diff>

<commit_message>
Update translation report with 2026-04-19 data
</commit_message>
<xml_diff>
--- a/reports/translation_jobs_all_days.xlsx
+++ b/reports/translation_jobs_all_days.xlsx
@@ -27515,7 +27515,7 @@
         <v>8166</v>
       </c>
       <c r="C2" s="7" t="n">
-        <v>18508</v>
+        <v>27289</v>
       </c>
       <c r="D2" s="7" t="n">
         <v>27289</v>
@@ -27531,7 +27531,7 @@
         <v>3</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D3" s="6" t="n">
         <v>1</v>
@@ -27547,7 +27547,7 @@
         <v>16</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>5</v>
@@ -27562,9 +27562,7 @@
       <c r="B5" s="7" t="n">
         <v>290</v>
       </c>
-      <c r="C5" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="C5" s="6" t="inlineStr"/>
       <c r="D5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
@@ -27577,7 +27575,7 @@
         <v>144</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>134</v>
@@ -27593,7 +27591,7 @@
         <v>2</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>4</v>
@@ -27609,7 +27607,7 @@
         <v>12</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>4</v>
@@ -27625,7 +27623,7 @@
         <v>136000</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>139429</v>
+        <v>146966</v>
       </c>
       <c r="D9" s="7" t="n">
         <v>146966</v>
@@ -27641,7 +27639,7 @@
         <v>334</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>6990</v>
+        <v>7311</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>7311</v>
@@ -27657,7 +27655,7 @@
         <v>11062</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>12280</v>
+        <v>12452</v>
       </c>
       <c r="D11" s="7" t="n">
         <v>12452</v>
@@ -27673,7 +27671,7 @@
         <v>1618</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>987</v>
+        <v>1342</v>
       </c>
       <c r="D12" s="7" t="n">
         <v>1342</v>
@@ -27689,7 +27687,7 @@
         <v>2911</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>2333</v>
+        <v>3177</v>
       </c>
       <c r="D13" s="7" t="n">
         <v>3177</v>
@@ -27705,7 +27703,7 @@
         <v>357</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>198</v>
+        <v>122</v>
       </c>
       <c r="D14" s="7" t="n">
         <v>122</v>
@@ -27817,16 +27815,16 @@
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>620</v>
+        <v>971</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>124</v>
+        <v>194</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>124</v>
+        <v>194</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>124</v>
+        <v>194</v>
       </c>
       <c r="F3" s="6" t="n">
         <v>0</v>

</xml_diff>